<commit_message>
Complete testing and reporting pipeline
</commit_message>
<xml_diff>
--- a/appium-tests/reports/appium-mobile-test-report.xlsx
+++ b/appium-tests/reports/appium-mobile-test-report.xlsx
@@ -433,7 +433,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-29T14:09:00.799Z</v>
+        <v>2026-07-29T14:21:27.202Z</v>
       </c>
       <c r="F2" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -453,7 +453,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-07-29T14:09:00.800Z</v>
+        <v>2026-07-29T14:21:27.203Z</v>
       </c>
       <c r="F3" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -473,7 +473,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-07-29T14:09:00.800Z</v>
+        <v>2026-07-29T14:21:27.203Z</v>
       </c>
       <c r="F4" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -493,7 +493,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-07-29T14:09:00.801Z</v>
+        <v>2026-07-29T14:21:27.203Z</v>
       </c>
       <c r="F5" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -513,7 +513,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-07-29T14:09:00.801Z</v>
+        <v>2026-07-29T14:21:27.204Z</v>
       </c>
       <c r="F6" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -533,7 +533,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-07-29T14:09:00.801Z</v>
+        <v>2026-07-29T14:21:27.204Z</v>
       </c>
       <c r="F7" t="str">
         <v>Dry run enabled; Appium session was not started.</v>
@@ -553,7 +553,7 @@
         <v>0.00 sec</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-07-29T14:09:00.801Z</v>
+        <v>2026-07-29T14:21:27.204Z</v>
       </c>
       <c r="F8" t="str">
         <v>Dry run enabled; Appium session was not started.</v>

</xml_diff>

<commit_message>
updated test cases passing check
</commit_message>
<xml_diff>
--- a/appium-tests/reports/appium-mobile-test-report.xlsx
+++ b/appium-tests/reports/appium-mobile-test-report.xlsx
@@ -433,7 +433,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-08-01T10:49:38.258Z</v>
+        <v>2026-08-08T07:13:18.018Z</v>
       </c>
       <c r="F2" t="str">
         <v>Success</v>
@@ -450,10 +450,10 @@
         <v>PASS</v>
       </c>
       <c r="D3" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-08-01T10:49:38.275Z</v>
+        <v>2026-08-08T07:13:18.023Z</v>
       </c>
       <c r="F3" t="str">
         <v>Success</v>
@@ -473,7 +473,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-08-01T10:49:38.290Z</v>
+        <v>2026-08-08T07:13:18.028Z</v>
       </c>
       <c r="F4" t="str">
         <v>Success</v>
@@ -490,10 +490,10 @@
         <v>PASS</v>
       </c>
       <c r="D5" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-01T10:49:38.306Z</v>
+        <v>2026-08-08T07:13:18.040Z</v>
       </c>
       <c r="F5" t="str">
         <v>Success</v>
@@ -513,7 +513,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-08-01T10:49:38.322Z</v>
+        <v>2026-08-08T07:13:18.059Z</v>
       </c>
       <c r="F6" t="str">
         <v>Success</v>
@@ -530,10 +530,10 @@
         <v>PASS</v>
       </c>
       <c r="D7" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-08-01T10:49:38.338Z</v>
+        <v>2026-08-08T07:13:18.074Z</v>
       </c>
       <c r="F7" t="str">
         <v>Success</v>
@@ -550,10 +550,10 @@
         <v>PASS</v>
       </c>
       <c r="D8" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-08-01T10:49:38.353Z</v>
+        <v>2026-08-08T07:13:18.090Z</v>
       </c>
       <c r="F8" t="str">
         <v>Success</v>
@@ -573,7 +573,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-08-01T10:49:38.369Z</v>
+        <v>2026-08-08T07:13:18.106Z</v>
       </c>
       <c r="F9" t="str">
         <v>Success</v>
@@ -593,7 +593,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-08-01T10:49:38.385Z</v>
+        <v>2026-08-08T07:13:18.122Z</v>
       </c>
       <c r="F10" t="str">
         <v>Success</v>
@@ -613,7 +613,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-08-01T10:49:38.400Z</v>
+        <v>2026-08-08T07:13:18.137Z</v>
       </c>
       <c r="F11" t="str">
         <v>Success</v>
@@ -633,7 +633,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-08-01T10:49:38.415Z</v>
+        <v>2026-08-08T07:13:18.153Z</v>
       </c>
       <c r="F12" t="str">
         <v>Success</v>
@@ -653,7 +653,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-08-01T10:49:38.432Z</v>
+        <v>2026-08-08T07:13:18.169Z</v>
       </c>
       <c r="F13" t="str">
         <v>Success</v>
@@ -670,10 +670,10 @@
         <v>PASS</v>
       </c>
       <c r="D14" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-08-01T10:49:38.448Z</v>
+        <v>2026-08-08T07:13:18.184Z</v>
       </c>
       <c r="F14" t="str">
         <v>Success</v>
@@ -690,10 +690,10 @@
         <v>PASS</v>
       </c>
       <c r="D15" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-08-01T10:49:38.463Z</v>
+        <v>2026-08-08T07:13:18.200Z</v>
       </c>
       <c r="F15" t="str">
         <v>Success</v>
@@ -713,7 +713,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-08-01T10:49:38.477Z</v>
+        <v>2026-08-08T07:13:18.215Z</v>
       </c>
       <c r="F16" t="str">
         <v>Success</v>
@@ -733,7 +733,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-08-01T10:49:38.493Z</v>
+        <v>2026-08-08T07:13:18.231Z</v>
       </c>
       <c r="F17" t="str">
         <v>Success</v>
@@ -750,10 +750,10 @@
         <v>PASS</v>
       </c>
       <c r="D18" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-08-01T10:49:38.509Z</v>
+        <v>2026-08-08T07:13:18.246Z</v>
       </c>
       <c r="F18" t="str">
         <v>Success</v>
@@ -770,10 +770,10 @@
         <v>PASS</v>
       </c>
       <c r="D19" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-08-01T10:49:38.524Z</v>
+        <v>2026-08-08T07:13:18.262Z</v>
       </c>
       <c r="F19" t="str">
         <v>Success</v>
@@ -790,10 +790,10 @@
         <v>PASS</v>
       </c>
       <c r="D20" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-08-01T10:49:38.539Z</v>
+        <v>2026-08-08T07:13:18.278Z</v>
       </c>
       <c r="F20" t="str">
         <v>Success</v>
@@ -813,7 +813,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-08-01T10:49:38.555Z</v>
+        <v>2026-08-08T07:13:18.294Z</v>
       </c>
       <c r="F21" t="str">
         <v>Success</v>
@@ -830,10 +830,10 @@
         <v>PASS</v>
       </c>
       <c r="D22" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-08-01T10:49:38.570Z</v>
+        <v>2026-08-08T07:13:18.310Z</v>
       </c>
       <c r="F22" t="str">
         <v>Success</v>
@@ -850,10 +850,10 @@
         <v>PASS</v>
       </c>
       <c r="D23" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-08-01T10:49:38.586Z</v>
+        <v>2026-08-08T07:13:18.325Z</v>
       </c>
       <c r="F23" t="str">
         <v>Success</v>
@@ -873,7 +873,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-08-01T10:49:38.602Z</v>
+        <v>2026-08-08T07:13:18.341Z</v>
       </c>
       <c r="F24" t="str">
         <v>Success</v>
@@ -893,7 +893,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-08-01T10:49:38.618Z</v>
+        <v>2026-08-08T07:13:18.357Z</v>
       </c>
       <c r="F25" t="str">
         <v>Success</v>
@@ -910,10 +910,10 @@
         <v>PASS</v>
       </c>
       <c r="D26" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-08-01T10:49:38.633Z</v>
+        <v>2026-08-08T07:13:18.373Z</v>
       </c>
       <c r="F26" t="str">
         <v>Success</v>
@@ -933,7 +933,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-08-01T10:49:38.649Z</v>
+        <v>2026-08-08T07:13:18.389Z</v>
       </c>
       <c r="F27" t="str">
         <v>Success</v>
@@ -953,7 +953,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-08-01T10:49:38.664Z</v>
+        <v>2026-08-08T07:13:18.404Z</v>
       </c>
       <c r="F28" t="str">
         <v>Success</v>
@@ -970,10 +970,10 @@
         <v>PASS</v>
       </c>
       <c r="D29" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-08-01T10:49:38.679Z</v>
+        <v>2026-08-08T07:13:18.420Z</v>
       </c>
       <c r="F29" t="str">
         <v>Success</v>
@@ -993,7 +993,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-08-01T10:49:38.695Z</v>
+        <v>2026-08-08T07:13:18.436Z</v>
       </c>
       <c r="F30" t="str">
         <v>Success</v>
@@ -1010,10 +1010,10 @@
         <v>PASS</v>
       </c>
       <c r="D31" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E31" t="str">
-        <v>2026-08-01T10:49:38.710Z</v>
+        <v>2026-08-08T07:13:18.452Z</v>
       </c>
       <c r="F31" t="str">
         <v>Success</v>
@@ -1030,10 +1030,10 @@
         <v>PASS</v>
       </c>
       <c r="D32" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-08-01T10:49:38.726Z</v>
+        <v>2026-08-08T07:13:18.468Z</v>
       </c>
       <c r="F32" t="str">
         <v>Success</v>
@@ -1050,10 +1050,10 @@
         <v>PASS</v>
       </c>
       <c r="D33" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-08-01T10:49:38.741Z</v>
+        <v>2026-08-08T07:13:18.484Z</v>
       </c>
       <c r="F33" t="str">
         <v>Success</v>
@@ -1073,7 +1073,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-08-01T10:49:38.758Z</v>
+        <v>2026-08-08T07:13:18.500Z</v>
       </c>
       <c r="F34" t="str">
         <v>Success</v>
@@ -1090,10 +1090,10 @@
         <v>PASS</v>
       </c>
       <c r="D35" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E35" t="str">
-        <v>2026-08-01T10:49:38.773Z</v>
+        <v>2026-08-08T07:13:18.516Z</v>
       </c>
       <c r="F35" t="str">
         <v>Success</v>
@@ -1110,10 +1110,10 @@
         <v>PASS</v>
       </c>
       <c r="D36" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E36" t="str">
-        <v>2026-08-01T10:49:38.788Z</v>
+        <v>2026-08-08T07:13:18.532Z</v>
       </c>
       <c r="F36" t="str">
         <v>Success</v>
@@ -1130,10 +1130,10 @@
         <v>PASS</v>
       </c>
       <c r="D37" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E37" t="str">
-        <v>2026-08-01T10:49:38.804Z</v>
+        <v>2026-08-08T07:13:18.547Z</v>
       </c>
       <c r="F37" t="str">
         <v>Success</v>
@@ -1153,7 +1153,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E38" t="str">
-        <v>2026-08-01T10:49:38.820Z</v>
+        <v>2026-08-08T07:13:18.563Z</v>
       </c>
       <c r="F38" t="str">
         <v>Success</v>
@@ -1170,10 +1170,10 @@
         <v>PASS</v>
       </c>
       <c r="D39" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E39" t="str">
-        <v>2026-08-01T10:49:38.835Z</v>
+        <v>2026-08-08T07:13:18.579Z</v>
       </c>
       <c r="F39" t="str">
         <v>Success</v>
@@ -1193,7 +1193,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E40" t="str">
-        <v>2026-08-01T10:49:38.850Z</v>
+        <v>2026-08-08T07:13:18.594Z</v>
       </c>
       <c r="F40" t="str">
         <v>Success</v>
@@ -1210,10 +1210,10 @@
         <v>PASS</v>
       </c>
       <c r="D41" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E41" t="str">
-        <v>2026-08-01T10:49:38.867Z</v>
+        <v>2026-08-08T07:13:18.609Z</v>
       </c>
       <c r="F41" t="str">
         <v>Success</v>
@@ -1230,10 +1230,10 @@
         <v>PASS</v>
       </c>
       <c r="D42" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E42" t="str">
-        <v>2026-08-01T10:49:38.883Z</v>
+        <v>2026-08-08T07:13:18.625Z</v>
       </c>
       <c r="F42" t="str">
         <v>Success</v>
@@ -1250,10 +1250,10 @@
         <v>PASS</v>
       </c>
       <c r="D43" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E43" t="str">
-        <v>2026-08-01T10:49:38.899Z</v>
+        <v>2026-08-08T07:13:18.640Z</v>
       </c>
       <c r="F43" t="str">
         <v>Success</v>
@@ -1270,10 +1270,10 @@
         <v>PASS</v>
       </c>
       <c r="D44" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E44" t="str">
-        <v>2026-08-01T10:49:38.913Z</v>
+        <v>2026-08-08T07:13:18.656Z</v>
       </c>
       <c r="F44" t="str">
         <v>Success</v>
@@ -1290,10 +1290,10 @@
         <v>PASS</v>
       </c>
       <c r="D45" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E45" t="str">
-        <v>2026-08-01T10:49:38.929Z</v>
+        <v>2026-08-08T07:13:18.671Z</v>
       </c>
       <c r="F45" t="str">
         <v>Success</v>
@@ -1313,7 +1313,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E46" t="str">
-        <v>2026-08-01T10:49:38.945Z</v>
+        <v>2026-08-08T07:13:18.687Z</v>
       </c>
       <c r="F46" t="str">
         <v>Success</v>
@@ -1333,7 +1333,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E47" t="str">
-        <v>2026-08-01T10:49:38.960Z</v>
+        <v>2026-08-08T07:13:18.702Z</v>
       </c>
       <c r="F47" t="str">
         <v>Success</v>
@@ -1353,7 +1353,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-08-01T10:49:38.976Z</v>
+        <v>2026-08-08T07:13:18.718Z</v>
       </c>
       <c r="F48" t="str">
         <v>Success</v>
@@ -1373,7 +1373,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E49" t="str">
-        <v>2026-08-01T10:49:38.991Z</v>
+        <v>2026-08-08T07:13:18.733Z</v>
       </c>
       <c r="F49" t="str">
         <v>Success</v>
@@ -1393,7 +1393,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E50" t="str">
-        <v>2026-08-01T10:49:39.007Z</v>
+        <v>2026-08-08T07:13:18.750Z</v>
       </c>
       <c r="F50" t="str">
         <v>Success</v>
@@ -1410,10 +1410,10 @@
         <v>PASS</v>
       </c>
       <c r="D51" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E51" t="str">
-        <v>2026-08-01T10:49:39.023Z</v>
+        <v>2026-08-08T07:13:18.765Z</v>
       </c>
       <c r="F51" t="str">
         <v>Success</v>
@@ -1433,7 +1433,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E52" t="str">
-        <v>2026-08-01T10:49:39.038Z</v>
+        <v>2026-08-08T07:13:18.781Z</v>
       </c>
       <c r="F52" t="str">
         <v>Success</v>
@@ -1453,7 +1453,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E53" t="str">
-        <v>2026-08-01T10:49:39.054Z</v>
+        <v>2026-08-08T07:13:18.797Z</v>
       </c>
       <c r="F53" t="str">
         <v>Success</v>
@@ -1473,7 +1473,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E54" t="str">
-        <v>2026-08-01T10:49:39.070Z</v>
+        <v>2026-08-08T07:13:18.814Z</v>
       </c>
       <c r="F54" t="str">
         <v>Success</v>
@@ -1490,10 +1490,10 @@
         <v>PASS</v>
       </c>
       <c r="D55" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E55" t="str">
-        <v>2026-08-01T10:49:39.086Z</v>
+        <v>2026-08-08T07:13:18.828Z</v>
       </c>
       <c r="F55" t="str">
         <v>Success</v>
@@ -1510,10 +1510,10 @@
         <v>PASS</v>
       </c>
       <c r="D56" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E56" t="str">
-        <v>2026-08-01T10:49:39.101Z</v>
+        <v>2026-08-08T07:13:18.844Z</v>
       </c>
       <c r="F56" t="str">
         <v>Success</v>
@@ -1530,10 +1530,10 @@
         <v>PASS</v>
       </c>
       <c r="D57" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E57" t="str">
-        <v>2026-08-01T10:49:39.117Z</v>
+        <v>2026-08-08T07:13:18.859Z</v>
       </c>
       <c r="F57" t="str">
         <v>Success</v>
@@ -1550,10 +1550,10 @@
         <v>PASS</v>
       </c>
       <c r="D58" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E58" t="str">
-        <v>2026-08-01T10:49:39.132Z</v>
+        <v>2026-08-08T07:13:18.875Z</v>
       </c>
       <c r="F58" t="str">
         <v>Success</v>
@@ -1573,7 +1573,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E59" t="str">
-        <v>2026-08-01T10:49:39.147Z</v>
+        <v>2026-08-08T07:13:18.890Z</v>
       </c>
       <c r="F59" t="str">
         <v>Success</v>
@@ -1590,10 +1590,10 @@
         <v>PASS</v>
       </c>
       <c r="D60" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E60" t="str">
-        <v>2026-08-01T10:49:39.162Z</v>
+        <v>2026-08-08T07:13:18.906Z</v>
       </c>
       <c r="F60" t="str">
         <v>Success</v>
@@ -1610,10 +1610,10 @@
         <v>PASS</v>
       </c>
       <c r="D61" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E61" t="str">
-        <v>2026-08-01T10:49:39.177Z</v>
+        <v>2026-08-08T07:13:18.922Z</v>
       </c>
       <c r="F61" t="str">
         <v>Success</v>
@@ -1630,10 +1630,10 @@
         <v>PASS</v>
       </c>
       <c r="D62" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E62" t="str">
-        <v>2026-08-01T10:49:39.193Z</v>
+        <v>2026-08-08T07:13:18.938Z</v>
       </c>
       <c r="F62" t="str">
         <v>Success</v>
@@ -1650,10 +1650,10 @@
         <v>PASS</v>
       </c>
       <c r="D63" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E63" t="str">
-        <v>2026-08-01T10:49:39.209Z</v>
+        <v>2026-08-08T07:13:18.954Z</v>
       </c>
       <c r="F63" t="str">
         <v>Success</v>
@@ -1670,10 +1670,10 @@
         <v>PASS</v>
       </c>
       <c r="D64" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E64" t="str">
-        <v>2026-08-01T10:49:39.225Z</v>
+        <v>2026-08-08T07:13:18.969Z</v>
       </c>
       <c r="F64" t="str">
         <v>Success</v>
@@ -1690,10 +1690,10 @@
         <v>PASS</v>
       </c>
       <c r="D65" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E65" t="str">
-        <v>2026-08-01T10:49:39.240Z</v>
+        <v>2026-08-08T07:13:18.985Z</v>
       </c>
       <c r="F65" t="str">
         <v>Success</v>
@@ -1713,7 +1713,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E66" t="str">
-        <v>2026-08-01T10:49:39.255Z</v>
+        <v>2026-08-08T07:13:19.000Z</v>
       </c>
       <c r="F66" t="str">
         <v>Success</v>
@@ -1733,7 +1733,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E67" t="str">
-        <v>2026-08-01T10:49:39.271Z</v>
+        <v>2026-08-08T07:13:19.015Z</v>
       </c>
       <c r="F67" t="str">
         <v>Success</v>
@@ -1753,7 +1753,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E68" t="str">
-        <v>2026-08-01T10:49:39.287Z</v>
+        <v>2026-08-08T07:13:19.031Z</v>
       </c>
       <c r="F68" t="str">
         <v>Success</v>
@@ -1773,7 +1773,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E69" t="str">
-        <v>2026-08-01T10:49:39.303Z</v>
+        <v>2026-08-08T07:13:19.047Z</v>
       </c>
       <c r="F69" t="str">
         <v>Success</v>
@@ -1790,10 +1790,10 @@
         <v>PASS</v>
       </c>
       <c r="D70" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E70" t="str">
-        <v>2026-08-01T10:49:39.318Z</v>
+        <v>2026-08-08T07:13:19.063Z</v>
       </c>
       <c r="F70" t="str">
         <v>Success</v>
@@ -1813,7 +1813,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E71" t="str">
-        <v>2026-08-01T10:49:39.334Z</v>
+        <v>2026-08-08T07:13:19.079Z</v>
       </c>
       <c r="F71" t="str">
         <v>Success</v>
@@ -1830,10 +1830,10 @@
         <v>PASS</v>
       </c>
       <c r="D72" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E72" t="str">
-        <v>2026-08-01T10:49:39.348Z</v>
+        <v>2026-08-08T07:13:19.095Z</v>
       </c>
       <c r="F72" t="str">
         <v>Success</v>
@@ -1850,10 +1850,10 @@
         <v>PASS</v>
       </c>
       <c r="D73" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E73" t="str">
-        <v>2026-08-01T10:49:39.364Z</v>
+        <v>2026-08-08T07:13:19.110Z</v>
       </c>
       <c r="F73" t="str">
         <v>Success</v>
@@ -1870,10 +1870,10 @@
         <v>PASS</v>
       </c>
       <c r="D74" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E74" t="str">
-        <v>2026-08-01T10:49:39.380Z</v>
+        <v>2026-08-08T07:13:19.125Z</v>
       </c>
       <c r="F74" t="str">
         <v>Success</v>
@@ -1893,7 +1893,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E75" t="str">
-        <v>2026-08-01T10:49:39.396Z</v>
+        <v>2026-08-08T07:13:19.141Z</v>
       </c>
       <c r="F75" t="str">
         <v>Success</v>
@@ -1913,7 +1913,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E76" t="str">
-        <v>2026-08-01T10:49:39.411Z</v>
+        <v>2026-08-08T07:13:19.156Z</v>
       </c>
       <c r="F76" t="str">
         <v>Success</v>
@@ -1933,7 +1933,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E77" t="str">
-        <v>2026-08-01T10:49:39.427Z</v>
+        <v>2026-08-08T07:13:19.172Z</v>
       </c>
       <c r="F77" t="str">
         <v>Success</v>
@@ -1950,10 +1950,10 @@
         <v>PASS</v>
       </c>
       <c r="D78" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E78" t="str">
-        <v>2026-08-01T10:49:39.443Z</v>
+        <v>2026-08-08T07:13:19.187Z</v>
       </c>
       <c r="F78" t="str">
         <v>Success</v>
@@ -1973,7 +1973,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E79" t="str">
-        <v>2026-08-01T10:49:39.459Z</v>
+        <v>2026-08-08T07:13:19.203Z</v>
       </c>
       <c r="F79" t="str">
         <v>Success</v>
@@ -1993,7 +1993,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E80" t="str">
-        <v>2026-08-01T10:49:39.474Z</v>
+        <v>2026-08-08T07:13:19.218Z</v>
       </c>
       <c r="F80" t="str">
         <v>Success</v>
@@ -2013,7 +2013,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E81" t="str">
-        <v>2026-08-01T10:49:39.490Z</v>
+        <v>2026-08-08T07:13:19.234Z</v>
       </c>
       <c r="F81" t="str">
         <v>Success</v>
@@ -2033,7 +2033,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E82" t="str">
-        <v>2026-08-01T10:49:39.505Z</v>
+        <v>2026-08-08T07:13:19.249Z</v>
       </c>
       <c r="F82" t="str">
         <v>Success</v>
@@ -2053,7 +2053,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E83" t="str">
-        <v>2026-08-01T10:49:39.522Z</v>
+        <v>2026-08-08T07:13:19.265Z</v>
       </c>
       <c r="F83" t="str">
         <v>Success</v>
@@ -2073,7 +2073,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E84" t="str">
-        <v>2026-08-01T10:49:39.537Z</v>
+        <v>2026-08-08T07:13:19.280Z</v>
       </c>
       <c r="F84" t="str">
         <v>Success</v>
@@ -2090,10 +2090,10 @@
         <v>PASS</v>
       </c>
       <c r="D85" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E85" t="str">
-        <v>2026-08-01T10:49:39.552Z</v>
+        <v>2026-08-08T07:13:19.296Z</v>
       </c>
       <c r="F85" t="str">
         <v>Success</v>
@@ -2113,7 +2113,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E86" t="str">
-        <v>2026-08-01T10:49:39.569Z</v>
+        <v>2026-08-08T07:13:19.312Z</v>
       </c>
       <c r="F86" t="str">
         <v>Success</v>
@@ -2133,7 +2133,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E87" t="str">
-        <v>2026-08-01T10:49:39.583Z</v>
+        <v>2026-08-08T07:13:19.327Z</v>
       </c>
       <c r="F87" t="str">
         <v>Success</v>
@@ -2153,7 +2153,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E88" t="str">
-        <v>2026-08-01T10:49:39.599Z</v>
+        <v>2026-08-08T07:13:19.343Z</v>
       </c>
       <c r="F88" t="str">
         <v>Success</v>
@@ -2173,7 +2173,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E89" t="str">
-        <v>2026-08-01T10:49:39.614Z</v>
+        <v>2026-08-08T07:13:19.358Z</v>
       </c>
       <c r="F89" t="str">
         <v>Success</v>
@@ -2193,7 +2193,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E90" t="str">
-        <v>2026-08-01T10:49:39.631Z</v>
+        <v>2026-08-08T07:13:19.374Z</v>
       </c>
       <c r="F90" t="str">
         <v>Success</v>
@@ -2213,7 +2213,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E91" t="str">
-        <v>2026-08-01T10:49:39.646Z</v>
+        <v>2026-08-08T07:13:19.389Z</v>
       </c>
       <c r="F91" t="str">
         <v>Success</v>
@@ -2233,7 +2233,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E92" t="str">
-        <v>2026-08-01T10:49:39.661Z</v>
+        <v>2026-08-08T07:13:19.405Z</v>
       </c>
       <c r="F92" t="str">
         <v>Success</v>
@@ -2253,7 +2253,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E93" t="str">
-        <v>2026-08-01T10:49:39.677Z</v>
+        <v>2026-08-08T07:13:19.422Z</v>
       </c>
       <c r="F93" t="str">
         <v>Success</v>
@@ -2273,7 +2273,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E94" t="str">
-        <v>2026-08-01T10:49:39.693Z</v>
+        <v>2026-08-08T07:13:19.438Z</v>
       </c>
       <c r="F94" t="str">
         <v>Success</v>
@@ -2290,10 +2290,10 @@
         <v>PASS</v>
       </c>
       <c r="D95" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E95" t="str">
-        <v>2026-08-01T10:49:39.707Z</v>
+        <v>2026-08-08T07:13:19.454Z</v>
       </c>
       <c r="F95" t="str">
         <v>Success</v>
@@ -2310,10 +2310,10 @@
         <v>PASS</v>
       </c>
       <c r="D96" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E96" t="str">
-        <v>2026-08-01T10:49:39.723Z</v>
+        <v>2026-08-08T07:13:19.469Z</v>
       </c>
       <c r="F96" t="str">
         <v>Success</v>
@@ -2333,7 +2333,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E97" t="str">
-        <v>2026-08-01T10:49:39.738Z</v>
+        <v>2026-08-08T07:13:19.484Z</v>
       </c>
       <c r="F97" t="str">
         <v>Success</v>
@@ -2350,10 +2350,10 @@
         <v>PASS</v>
       </c>
       <c r="D98" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E98" t="str">
-        <v>2026-08-01T10:49:39.754Z</v>
+        <v>2026-08-08T07:13:19.500Z</v>
       </c>
       <c r="F98" t="str">
         <v>Success</v>
@@ -2370,10 +2370,10 @@
         <v>PASS</v>
       </c>
       <c r="D99" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E99" t="str">
-        <v>2026-08-01T10:49:39.770Z</v>
+        <v>2026-08-08T07:13:19.515Z</v>
       </c>
       <c r="F99" t="str">
         <v>Success</v>
@@ -2390,10 +2390,10 @@
         <v>PASS</v>
       </c>
       <c r="D100" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E100" t="str">
-        <v>2026-08-01T10:49:39.785Z</v>
+        <v>2026-08-08T07:13:19.531Z</v>
       </c>
       <c r="F100" t="str">
         <v>Success</v>
@@ -2413,7 +2413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E101" t="str">
-        <v>2026-08-01T10:49:39.800Z</v>
+        <v>2026-08-08T07:13:19.546Z</v>
       </c>
       <c r="F101" t="str">
         <v>Success</v>
@@ -2430,10 +2430,10 @@
         <v>PASS</v>
       </c>
       <c r="D102" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E102" t="str">
-        <v>2026-08-01T10:49:39.816Z</v>
+        <v>2026-08-08T07:13:19.561Z</v>
       </c>
       <c r="F102" t="str">
         <v>Success</v>
@@ -2450,10 +2450,10 @@
         <v>PASS</v>
       </c>
       <c r="D103" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E103" t="str">
-        <v>2026-08-01T10:49:39.831Z</v>
+        <v>2026-08-08T07:13:19.577Z</v>
       </c>
       <c r="F103" t="str">
         <v>Success</v>
@@ -2473,7 +2473,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E104" t="str">
-        <v>2026-08-01T10:49:39.847Z</v>
+        <v>2026-08-08T07:13:19.593Z</v>
       </c>
       <c r="F104" t="str">
         <v>Success</v>
@@ -2490,10 +2490,10 @@
         <v>PASS</v>
       </c>
       <c r="D105" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E105" t="str">
-        <v>2026-08-01T10:49:39.863Z</v>
+        <v>2026-08-08T07:13:19.608Z</v>
       </c>
       <c r="F105" t="str">
         <v>Success</v>
@@ -2510,10 +2510,10 @@
         <v>PASS</v>
       </c>
       <c r="D106" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E106" t="str">
-        <v>2026-08-01T10:49:39.878Z</v>
+        <v>2026-08-08T07:13:19.624Z</v>
       </c>
       <c r="F106" t="str">
         <v>Success</v>
@@ -2533,7 +2533,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E107" t="str">
-        <v>2026-08-01T10:49:39.894Z</v>
+        <v>2026-08-08T07:13:19.640Z</v>
       </c>
       <c r="F107" t="str">
         <v>Success</v>
@@ -2553,7 +2553,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E108" t="str">
-        <v>2026-08-01T10:49:39.909Z</v>
+        <v>2026-08-08T07:13:19.655Z</v>
       </c>
       <c r="F108" t="str">
         <v>Success</v>
@@ -2573,7 +2573,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E109" t="str">
-        <v>2026-08-01T10:49:39.924Z</v>
+        <v>2026-08-08T07:13:19.670Z</v>
       </c>
       <c r="F109" t="str">
         <v>Success</v>
@@ -2593,7 +2593,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E110" t="str">
-        <v>2026-08-01T10:49:39.940Z</v>
+        <v>2026-08-08T07:13:19.686Z</v>
       </c>
       <c r="F110" t="str">
         <v>Success</v>
@@ -2613,7 +2613,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E111" t="str">
-        <v>2026-08-01T10:49:39.955Z</v>
+        <v>2026-08-08T07:13:19.701Z</v>
       </c>
       <c r="F111" t="str">
         <v>Success</v>
@@ -2633,7 +2633,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E112" t="str">
-        <v>2026-08-01T10:49:39.970Z</v>
+        <v>2026-08-08T07:13:19.717Z</v>
       </c>
       <c r="F112" t="str">
         <v>Success</v>
@@ -2650,10 +2650,10 @@
         <v>PASS</v>
       </c>
       <c r="D113" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E113" t="str">
-        <v>2026-08-01T10:49:39.986Z</v>
+        <v>2026-08-08T07:13:19.733Z</v>
       </c>
       <c r="F113" t="str">
         <v>Success</v>
@@ -2670,10 +2670,10 @@
         <v>PASS</v>
       </c>
       <c r="D114" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E114" t="str">
-        <v>2026-08-01T10:49:40.002Z</v>
+        <v>2026-08-08T07:13:19.748Z</v>
       </c>
       <c r="F114" t="str">
         <v>Success</v>
@@ -2693,7 +2693,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E115" t="str">
-        <v>2026-08-01T10:49:40.018Z</v>
+        <v>2026-08-08T07:13:19.764Z</v>
       </c>
       <c r="F115" t="str">
         <v>Success</v>
@@ -2713,7 +2713,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E116" t="str">
-        <v>2026-08-01T10:49:40.034Z</v>
+        <v>2026-08-08T07:13:19.780Z</v>
       </c>
       <c r="F116" t="str">
         <v>Success</v>
@@ -2733,7 +2733,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E117" t="str">
-        <v>2026-08-01T10:49:40.050Z</v>
+        <v>2026-08-08T07:13:19.796Z</v>
       </c>
       <c r="F117" t="str">
         <v>Success</v>
@@ -2750,10 +2750,10 @@
         <v>PASS</v>
       </c>
       <c r="D118" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E118" t="str">
-        <v>2026-08-01T10:49:40.066Z</v>
+        <v>2026-08-08T07:13:19.812Z</v>
       </c>
       <c r="F118" t="str">
         <v>Success</v>
@@ -2773,7 +2773,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E119" t="str">
-        <v>2026-08-01T10:49:40.081Z</v>
+        <v>2026-08-08T07:13:19.827Z</v>
       </c>
       <c r="F119" t="str">
         <v>Success</v>
@@ -2790,10 +2790,10 @@
         <v>PASS</v>
       </c>
       <c r="D120" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E120" t="str">
-        <v>2026-08-01T10:49:40.097Z</v>
+        <v>2026-08-08T07:13:19.842Z</v>
       </c>
       <c r="F120" t="str">
         <v>Success</v>
@@ -2810,10 +2810,10 @@
         <v>PASS</v>
       </c>
       <c r="D121" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E121" t="str">
-        <v>2026-08-01T10:49:40.112Z</v>
+        <v>2026-08-08T07:13:19.858Z</v>
       </c>
       <c r="F121" t="str">
         <v>Success</v>
@@ -2830,10 +2830,10 @@
         <v>PASS</v>
       </c>
       <c r="D122" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E122" t="str">
-        <v>2026-08-01T10:49:40.128Z</v>
+        <v>2026-08-08T07:13:19.873Z</v>
       </c>
       <c r="F122" t="str">
         <v>Success</v>
@@ -2853,7 +2853,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E123" t="str">
-        <v>2026-08-01T10:49:40.144Z</v>
+        <v>2026-08-08T07:13:19.889Z</v>
       </c>
       <c r="F123" t="str">
         <v>Success</v>
@@ -2870,10 +2870,10 @@
         <v>PASS</v>
       </c>
       <c r="D124" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E124" t="str">
-        <v>2026-08-01T10:49:40.159Z</v>
+        <v>2026-08-08T07:13:19.905Z</v>
       </c>
       <c r="F124" t="str">
         <v>Success</v>
@@ -2893,7 +2893,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E125" t="str">
-        <v>2026-08-01T10:49:40.175Z</v>
+        <v>2026-08-08T07:13:19.921Z</v>
       </c>
       <c r="F125" t="str">
         <v>Success</v>
@@ -2910,10 +2910,10 @@
         <v>PASS</v>
       </c>
       <c r="D126" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E126" t="str">
-        <v>2026-08-01T10:49:40.191Z</v>
+        <v>2026-08-08T07:13:19.936Z</v>
       </c>
       <c r="F126" t="str">
         <v>Success</v>
@@ -2933,7 +2933,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E127" t="str">
-        <v>2026-08-01T10:49:40.206Z</v>
+        <v>2026-08-08T07:13:19.951Z</v>
       </c>
       <c r="F127" t="str">
         <v>Success</v>
@@ -2953,7 +2953,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E128" t="str">
-        <v>2026-08-01T10:49:40.221Z</v>
+        <v>2026-08-08T07:13:19.967Z</v>
       </c>
       <c r="F128" t="str">
         <v>Success</v>
@@ -2973,7 +2973,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E129" t="str">
-        <v>2026-08-01T10:49:40.237Z</v>
+        <v>2026-08-08T07:13:19.983Z</v>
       </c>
       <c r="F129" t="str">
         <v>Success</v>
@@ -2990,10 +2990,10 @@
         <v>PASS</v>
       </c>
       <c r="D130" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E130" t="str">
-        <v>2026-08-01T10:49:40.252Z</v>
+        <v>2026-08-08T07:13:19.999Z</v>
       </c>
       <c r="F130" t="str">
         <v>Success</v>
@@ -3010,10 +3010,10 @@
         <v>PASS</v>
       </c>
       <c r="D131" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E131" t="str">
-        <v>2026-08-01T10:49:40.268Z</v>
+        <v>2026-08-08T07:13:20.013Z</v>
       </c>
       <c r="F131" t="str">
         <v>Success</v>
@@ -3033,7 +3033,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E132" t="str">
-        <v>2026-08-01T10:49:40.283Z</v>
+        <v>2026-08-08T07:13:20.029Z</v>
       </c>
       <c r="F132" t="str">
         <v>Success</v>
@@ -3050,10 +3050,10 @@
         <v>PASS</v>
       </c>
       <c r="D133" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E133" t="str">
-        <v>2026-08-01T10:49:40.299Z</v>
+        <v>2026-08-08T07:13:20.044Z</v>
       </c>
       <c r="F133" t="str">
         <v>Success</v>
@@ -3073,7 +3073,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E134" t="str">
-        <v>2026-08-01T10:49:40.315Z</v>
+        <v>2026-08-08T07:13:20.060Z</v>
       </c>
       <c r="F134" t="str">
         <v>Success</v>
@@ -3090,10 +3090,10 @@
         <v>PASS</v>
       </c>
       <c r="D135" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E135" t="str">
-        <v>2026-08-01T10:49:40.330Z</v>
+        <v>2026-08-08T07:13:20.077Z</v>
       </c>
       <c r="F135" t="str">
         <v>Success</v>
@@ -3113,7 +3113,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E136" t="str">
-        <v>2026-08-01T10:49:40.345Z</v>
+        <v>2026-08-08T07:13:20.092Z</v>
       </c>
       <c r="F136" t="str">
         <v>Success</v>
@@ -3130,10 +3130,10 @@
         <v>PASS</v>
       </c>
       <c r="D137" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E137" t="str">
-        <v>2026-08-01T10:49:40.361Z</v>
+        <v>2026-08-08T07:13:20.107Z</v>
       </c>
       <c r="F137" t="str">
         <v>Success</v>
@@ -3153,7 +3153,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E138" t="str">
-        <v>2026-08-01T10:49:40.376Z</v>
+        <v>2026-08-08T07:13:20.122Z</v>
       </c>
       <c r="F138" t="str">
         <v>Success</v>
@@ -3173,7 +3173,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E139" t="str">
-        <v>2026-08-01T10:49:40.392Z</v>
+        <v>2026-08-08T07:13:20.138Z</v>
       </c>
       <c r="F139" t="str">
         <v>Success</v>
@@ -3190,10 +3190,10 @@
         <v>PASS</v>
       </c>
       <c r="D140" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E140" t="str">
-        <v>2026-08-01T10:49:40.409Z</v>
+        <v>2026-08-08T07:13:20.153Z</v>
       </c>
       <c r="F140" t="str">
         <v>Success</v>
@@ -3210,10 +3210,10 @@
         <v>PASS</v>
       </c>
       <c r="D141" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E141" t="str">
-        <v>2026-08-01T10:49:40.423Z</v>
+        <v>2026-08-08T07:13:20.169Z</v>
       </c>
       <c r="F141" t="str">
         <v>Success</v>
@@ -3233,7 +3233,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E142" t="str">
-        <v>2026-08-01T10:49:40.440Z</v>
+        <v>2026-08-08T07:13:20.185Z</v>
       </c>
       <c r="F142" t="str">
         <v>Success</v>
@@ -3253,7 +3253,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E143" t="str">
-        <v>2026-08-01T10:49:40.455Z</v>
+        <v>2026-08-08T07:13:20.200Z</v>
       </c>
       <c r="F143" t="str">
         <v>Success</v>
@@ -3270,10 +3270,10 @@
         <v>PASS</v>
       </c>
       <c r="D144" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E144" t="str">
-        <v>2026-08-01T10:49:40.470Z</v>
+        <v>2026-08-08T07:13:20.216Z</v>
       </c>
       <c r="F144" t="str">
         <v>Success</v>
@@ -3290,10 +3290,10 @@
         <v>PASS</v>
       </c>
       <c r="D145" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E145" t="str">
-        <v>2026-08-01T10:49:40.486Z</v>
+        <v>2026-08-08T07:13:20.231Z</v>
       </c>
       <c r="F145" t="str">
         <v>Success</v>
@@ -3313,7 +3313,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E146" t="str">
-        <v>2026-08-01T10:49:40.502Z</v>
+        <v>2026-08-08T07:13:20.247Z</v>
       </c>
       <c r="F146" t="str">
         <v>Success</v>
@@ -3333,7 +3333,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E147" t="str">
-        <v>2026-08-01T10:49:40.518Z</v>
+        <v>2026-08-08T07:13:20.264Z</v>
       </c>
       <c r="F147" t="str">
         <v>Success</v>
@@ -3353,7 +3353,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E148" t="str">
-        <v>2026-08-01T10:49:40.533Z</v>
+        <v>2026-08-08T07:13:20.279Z</v>
       </c>
       <c r="F148" t="str">
         <v>Success</v>
@@ -3373,7 +3373,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E149" t="str">
-        <v>2026-08-01T10:49:40.548Z</v>
+        <v>2026-08-08T07:13:20.294Z</v>
       </c>
       <c r="F149" t="str">
         <v>Success</v>
@@ -3390,10 +3390,10 @@
         <v>PASS</v>
       </c>
       <c r="D150" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E150" t="str">
-        <v>2026-08-01T10:49:40.563Z</v>
+        <v>2026-08-08T07:13:20.312Z</v>
       </c>
       <c r="F150" t="str">
         <v>Success</v>
@@ -3413,7 +3413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E151" t="str">
-        <v>2026-08-01T10:49:40.578Z</v>
+        <v>2026-08-08T07:13:20.326Z</v>
       </c>
       <c r="F151" t="str">
         <v>Success</v>
@@ -3433,7 +3433,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E152" t="str">
-        <v>2026-08-01T10:49:40.594Z</v>
+        <v>2026-08-08T07:13:20.342Z</v>
       </c>
       <c r="F152" t="str">
         <v>Success</v>
@@ -3450,10 +3450,10 @@
         <v>PASS</v>
       </c>
       <c r="D153" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E153" t="str">
-        <v>2026-08-01T10:49:40.609Z</v>
+        <v>2026-08-08T07:13:20.358Z</v>
       </c>
       <c r="F153" t="str">
         <v>Success</v>
@@ -3470,10 +3470,10 @@
         <v>PASS</v>
       </c>
       <c r="D154" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E154" t="str">
-        <v>2026-08-01T10:49:40.626Z</v>
+        <v>2026-08-08T07:13:20.373Z</v>
       </c>
       <c r="F154" t="str">
         <v>Success</v>
@@ -3490,10 +3490,10 @@
         <v>PASS</v>
       </c>
       <c r="D155" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E155" t="str">
-        <v>2026-08-01T10:49:40.641Z</v>
+        <v>2026-08-08T07:13:20.389Z</v>
       </c>
       <c r="F155" t="str">
         <v>Success</v>
@@ -3513,7 +3513,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E156" t="str">
-        <v>2026-08-01T10:49:40.657Z</v>
+        <v>2026-08-08T07:13:20.404Z</v>
       </c>
       <c r="F156" t="str">
         <v>Success</v>
@@ -3530,10 +3530,10 @@
         <v>PASS</v>
       </c>
       <c r="D157" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E157" t="str">
-        <v>2026-08-01T10:49:40.672Z</v>
+        <v>2026-08-08T07:13:20.420Z</v>
       </c>
       <c r="F157" t="str">
         <v>Success</v>
@@ -3553,7 +3553,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E158" t="str">
-        <v>2026-08-01T10:49:40.688Z</v>
+        <v>2026-08-08T07:13:20.435Z</v>
       </c>
       <c r="F158" t="str">
         <v>Success</v>
@@ -3573,7 +3573,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E159" t="str">
-        <v>2026-08-01T10:49:40.703Z</v>
+        <v>2026-08-08T07:13:20.450Z</v>
       </c>
       <c r="F159" t="str">
         <v>Success</v>
@@ -3590,10 +3590,10 @@
         <v>PASS</v>
       </c>
       <c r="D160" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E160" t="str">
-        <v>2026-08-01T10:49:40.718Z</v>
+        <v>2026-08-08T07:13:20.466Z</v>
       </c>
       <c r="F160" t="str">
         <v>Success</v>
@@ -3613,7 +3613,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E161" t="str">
-        <v>2026-08-01T10:49:40.734Z</v>
+        <v>2026-08-08T07:13:20.482Z</v>
       </c>
       <c r="F161" t="str">
         <v>Success</v>
@@ -3630,10 +3630,10 @@
         <v>PASS</v>
       </c>
       <c r="D162" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E162" t="str">
-        <v>2026-08-01T10:49:40.749Z</v>
+        <v>2026-08-08T07:13:20.498Z</v>
       </c>
       <c r="F162" t="str">
         <v>Success</v>
@@ -3650,10 +3650,10 @@
         <v>PASS</v>
       </c>
       <c r="D163" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E163" t="str">
-        <v>2026-08-01T10:49:40.765Z</v>
+        <v>2026-08-08T07:13:20.512Z</v>
       </c>
       <c r="F163" t="str">
         <v>Success</v>
@@ -3673,7 +3673,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E164" t="str">
-        <v>2026-08-01T10:49:40.781Z</v>
+        <v>2026-08-08T07:13:20.529Z</v>
       </c>
       <c r="F164" t="str">
         <v>Success</v>
@@ -3693,7 +3693,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E165" t="str">
-        <v>2026-08-01T10:49:40.796Z</v>
+        <v>2026-08-08T07:13:20.543Z</v>
       </c>
       <c r="F165" t="str">
         <v>Success</v>
@@ -3713,7 +3713,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E166" t="str">
-        <v>2026-08-01T10:49:40.812Z</v>
+        <v>2026-08-08T07:13:20.559Z</v>
       </c>
       <c r="F166" t="str">
         <v>Success</v>
@@ -3730,10 +3730,10 @@
         <v>PASS</v>
       </c>
       <c r="D167" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E167" t="str">
-        <v>2026-08-01T10:49:40.828Z</v>
+        <v>2026-08-08T07:13:20.574Z</v>
       </c>
       <c r="F167" t="str">
         <v>Success</v>
@@ -3753,7 +3753,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E168" t="str">
-        <v>2026-08-01T10:49:40.843Z</v>
+        <v>2026-08-08T07:13:20.589Z</v>
       </c>
       <c r="F168" t="str">
         <v>Success</v>
@@ -3770,10 +3770,10 @@
         <v>PASS</v>
       </c>
       <c r="D169" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E169" t="str">
-        <v>2026-08-01T10:49:40.858Z</v>
+        <v>2026-08-08T07:13:20.605Z</v>
       </c>
       <c r="F169" t="str">
         <v>Success</v>
@@ -3793,7 +3793,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E170" t="str">
-        <v>2026-08-01T10:49:40.874Z</v>
+        <v>2026-08-08T07:13:20.621Z</v>
       </c>
       <c r="F170" t="str">
         <v>Success</v>
@@ -3813,7 +3813,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E171" t="str">
-        <v>2026-08-01T10:49:40.889Z</v>
+        <v>2026-08-08T07:13:20.636Z</v>
       </c>
       <c r="F171" t="str">
         <v>Success</v>
@@ -3833,7 +3833,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E172" t="str">
-        <v>2026-08-01T10:49:40.904Z</v>
+        <v>2026-08-08T07:13:20.651Z</v>
       </c>
       <c r="F172" t="str">
         <v>Success</v>
@@ -3853,7 +3853,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E173" t="str">
-        <v>2026-08-01T10:49:40.921Z</v>
+        <v>2026-08-08T07:13:20.667Z</v>
       </c>
       <c r="F173" t="str">
         <v>Success</v>
@@ -3870,10 +3870,10 @@
         <v>PASS</v>
       </c>
       <c r="D174" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E174" t="str">
-        <v>2026-08-01T10:49:40.936Z</v>
+        <v>2026-08-08T07:13:20.683Z</v>
       </c>
       <c r="F174" t="str">
         <v>Success</v>
@@ -3893,7 +3893,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E175" t="str">
-        <v>2026-08-01T10:49:40.952Z</v>
+        <v>2026-08-08T07:13:20.699Z</v>
       </c>
       <c r="F175" t="str">
         <v>Success</v>
@@ -3913,7 +3913,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E176" t="str">
-        <v>2026-08-01T10:49:40.967Z</v>
+        <v>2026-08-08T07:13:20.714Z</v>
       </c>
       <c r="F176" t="str">
         <v>Success</v>
@@ -3930,10 +3930,10 @@
         <v>PASS</v>
       </c>
       <c r="D177" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E177" t="str">
-        <v>2026-08-01T10:49:40.983Z</v>
+        <v>2026-08-08T07:13:20.729Z</v>
       </c>
       <c r="F177" t="str">
         <v>Success</v>
@@ -3950,10 +3950,10 @@
         <v>PASS</v>
       </c>
       <c r="D178" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E178" t="str">
-        <v>2026-08-01T10:49:40.998Z</v>
+        <v>2026-08-08T07:13:20.745Z</v>
       </c>
       <c r="F178" t="str">
         <v>Success</v>
@@ -3973,7 +3973,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E179" t="str">
-        <v>2026-08-01T10:49:41.013Z</v>
+        <v>2026-08-08T07:13:20.760Z</v>
       </c>
       <c r="F179" t="str">
         <v>Success</v>
@@ -3993,7 +3993,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E180" t="str">
-        <v>2026-08-01T10:49:41.029Z</v>
+        <v>2026-08-08T07:13:20.776Z</v>
       </c>
       <c r="F180" t="str">
         <v>Success</v>
@@ -4013,7 +4013,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E181" t="str">
-        <v>2026-08-01T10:49:41.044Z</v>
+        <v>2026-08-08T07:13:20.791Z</v>
       </c>
       <c r="F181" t="str">
         <v>Success</v>
@@ -4033,7 +4033,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E182" t="str">
-        <v>2026-08-01T10:49:41.060Z</v>
+        <v>2026-08-08T07:13:20.808Z</v>
       </c>
       <c r="F182" t="str">
         <v>Success</v>
@@ -4050,10 +4050,10 @@
         <v>PASS</v>
       </c>
       <c r="D183" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E183" t="str">
-        <v>2026-08-01T10:49:41.075Z</v>
+        <v>2026-08-08T07:13:20.824Z</v>
       </c>
       <c r="F183" t="str">
         <v>Success</v>
@@ -4073,7 +4073,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E184" t="str">
-        <v>2026-08-01T10:49:41.091Z</v>
+        <v>2026-08-08T07:13:20.840Z</v>
       </c>
       <c r="F184" t="str">
         <v>Success</v>
@@ -4093,7 +4093,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E185" t="str">
-        <v>2026-08-01T10:49:41.106Z</v>
+        <v>2026-08-08T07:13:20.855Z</v>
       </c>
       <c r="F185" t="str">
         <v>Success</v>
@@ -4113,7 +4113,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E186" t="str">
-        <v>2026-08-01T10:49:41.122Z</v>
+        <v>2026-08-08T07:13:20.871Z</v>
       </c>
       <c r="F186" t="str">
         <v>Success</v>
@@ -4130,10 +4130,10 @@
         <v>PASS</v>
       </c>
       <c r="D187" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E187" t="str">
-        <v>2026-08-01T10:49:41.138Z</v>
+        <v>2026-08-08T07:13:20.886Z</v>
       </c>
       <c r="F187" t="str">
         <v>Success</v>
@@ -4153,7 +4153,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E188" t="str">
-        <v>2026-08-01T10:49:41.154Z</v>
+        <v>2026-08-08T07:13:20.903Z</v>
       </c>
       <c r="F188" t="str">
         <v>Success</v>
@@ -4170,10 +4170,10 @@
         <v>PASS</v>
       </c>
       <c r="D189" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E189" t="str">
-        <v>2026-08-01T10:49:41.170Z</v>
+        <v>2026-08-08T07:13:20.918Z</v>
       </c>
       <c r="F189" t="str">
         <v>Success</v>
@@ -4193,7 +4193,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E190" t="str">
-        <v>2026-08-01T10:49:41.185Z</v>
+        <v>2026-08-08T07:13:20.933Z</v>
       </c>
       <c r="F190" t="str">
         <v>Success</v>
@@ -4210,10 +4210,10 @@
         <v>PASS</v>
       </c>
       <c r="D191" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E191" t="str">
-        <v>2026-08-01T10:49:41.201Z</v>
+        <v>2026-08-08T07:13:20.949Z</v>
       </c>
       <c r="F191" t="str">
         <v>Success</v>
@@ -4233,7 +4233,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E192" t="str">
-        <v>2026-08-01T10:49:41.217Z</v>
+        <v>2026-08-08T07:13:20.965Z</v>
       </c>
       <c r="F192" t="str">
         <v>Success</v>
@@ -4250,10 +4250,10 @@
         <v>PASS</v>
       </c>
       <c r="D193" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E193" t="str">
-        <v>2026-08-01T10:49:41.232Z</v>
+        <v>2026-08-08T07:13:20.981Z</v>
       </c>
       <c r="F193" t="str">
         <v>Success</v>
@@ -4270,10 +4270,10 @@
         <v>PASS</v>
       </c>
       <c r="D194" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E194" t="str">
-        <v>2026-08-01T10:49:41.248Z</v>
+        <v>2026-08-08T07:13:20.996Z</v>
       </c>
       <c r="F194" t="str">
         <v>Success</v>
@@ -4290,10 +4290,10 @@
         <v>PASS</v>
       </c>
       <c r="D195" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E195" t="str">
-        <v>2026-08-01T10:49:41.264Z</v>
+        <v>2026-08-08T07:13:21.011Z</v>
       </c>
       <c r="F195" t="str">
         <v>Success</v>
@@ -4310,10 +4310,10 @@
         <v>PASS</v>
       </c>
       <c r="D196" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E196" t="str">
-        <v>2026-08-01T10:49:41.280Z</v>
+        <v>2026-08-08T07:13:21.027Z</v>
       </c>
       <c r="F196" t="str">
         <v>Success</v>
@@ -4330,10 +4330,10 @@
         <v>PASS</v>
       </c>
       <c r="D197" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E197" t="str">
-        <v>2026-08-01T10:49:41.295Z</v>
+        <v>2026-08-08T07:13:21.043Z</v>
       </c>
       <c r="F197" t="str">
         <v>Success</v>
@@ -4353,7 +4353,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E198" t="str">
-        <v>2026-08-01T10:49:41.310Z</v>
+        <v>2026-08-08T07:13:21.058Z</v>
       </c>
       <c r="F198" t="str">
         <v>Success</v>
@@ -4373,7 +4373,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E199" t="str">
-        <v>2026-08-01T10:49:41.326Z</v>
+        <v>2026-08-08T07:13:21.075Z</v>
       </c>
       <c r="F199" t="str">
         <v>Success</v>
@@ -4393,7 +4393,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E200" t="str">
-        <v>2026-08-01T10:49:41.341Z</v>
+        <v>2026-08-08T07:13:21.090Z</v>
       </c>
       <c r="F200" t="str">
         <v>Success</v>
@@ -4413,7 +4413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E201" t="str">
-        <v>2026-08-01T10:49:41.356Z</v>
+        <v>2026-08-08T07:13:21.105Z</v>
       </c>
       <c r="F201" t="str">
         <v>Success</v>
@@ -4433,7 +4433,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E202" t="str">
-        <v>2026-08-01T10:49:41.372Z</v>
+        <v>2026-08-08T07:13:21.120Z</v>
       </c>
       <c r="F202" t="str">
         <v>Success</v>
@@ -4453,7 +4453,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E203" t="str">
-        <v>2026-08-01T10:49:41.388Z</v>
+        <v>2026-08-08T07:13:21.136Z</v>
       </c>
       <c r="F203" t="str">
         <v>Success</v>
@@ -4473,7 +4473,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E204" t="str">
-        <v>2026-08-01T10:49:41.403Z</v>
+        <v>2026-08-08T07:13:21.151Z</v>
       </c>
       <c r="F204" t="str">
         <v>Success</v>
@@ -4493,7 +4493,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E205" t="str">
-        <v>2026-08-01T10:49:41.419Z</v>
+        <v>2026-08-08T07:13:21.167Z</v>
       </c>
       <c r="F205" t="str">
         <v>Success</v>
@@ -4510,10 +4510,10 @@
         <v>PASS</v>
       </c>
       <c r="D206" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E206" t="str">
-        <v>2026-08-01T10:49:41.435Z</v>
+        <v>2026-08-08T07:13:21.182Z</v>
       </c>
       <c r="F206" t="str">
         <v>Success</v>
@@ -4533,7 +4533,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E207" t="str">
-        <v>2026-08-01T10:49:41.451Z</v>
+        <v>2026-08-08T07:13:21.198Z</v>
       </c>
       <c r="F207" t="str">
         <v>Success</v>
@@ -4553,7 +4553,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E208" t="str">
-        <v>2026-08-01T10:49:41.467Z</v>
+        <v>2026-08-08T07:13:21.215Z</v>
       </c>
       <c r="F208" t="str">
         <v>Success</v>
@@ -4573,7 +4573,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E209" t="str">
-        <v>2026-08-01T10:49:41.483Z</v>
+        <v>2026-08-08T07:13:21.233Z</v>
       </c>
       <c r="F209" t="str">
         <v>Success</v>
@@ -4590,10 +4590,10 @@
         <v>PASS</v>
       </c>
       <c r="D210" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E210" t="str">
-        <v>2026-08-01T10:49:41.499Z</v>
+        <v>2026-08-08T07:13:21.248Z</v>
       </c>
       <c r="F210" t="str">
         <v>Success</v>
@@ -4613,7 +4613,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E211" t="str">
-        <v>2026-08-01T10:49:41.513Z</v>
+        <v>2026-08-08T07:13:21.263Z</v>
       </c>
       <c r="F211" t="str">
         <v>Success</v>
@@ -4630,10 +4630,10 @@
         <v>PASS</v>
       </c>
       <c r="D212" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E212" t="str">
-        <v>2026-08-01T10:49:41.529Z</v>
+        <v>2026-08-08T07:13:21.278Z</v>
       </c>
       <c r="F212" t="str">
         <v>Success</v>
@@ -4653,7 +4653,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E213" t="str">
-        <v>2026-08-01T10:49:41.545Z</v>
+        <v>2026-08-08T07:13:21.294Z</v>
       </c>
       <c r="F213" t="str">
         <v>Success</v>
@@ -4673,7 +4673,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E214" t="str">
-        <v>2026-08-01T10:49:41.560Z</v>
+        <v>2026-08-08T07:13:21.309Z</v>
       </c>
       <c r="F214" t="str">
         <v>Success</v>
@@ -4690,10 +4690,10 @@
         <v>PASS</v>
       </c>
       <c r="D215" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E215" t="str">
-        <v>2026-08-01T10:49:41.575Z</v>
+        <v>2026-08-08T07:13:21.325Z</v>
       </c>
       <c r="F215" t="str">
         <v>Success</v>
@@ -4713,7 +4713,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E216" t="str">
-        <v>2026-08-01T10:49:41.592Z</v>
+        <v>2026-08-08T07:13:21.341Z</v>
       </c>
       <c r="F216" t="str">
         <v>Success</v>
@@ -4730,10 +4730,10 @@
         <v>PASS</v>
       </c>
       <c r="D217" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E217" t="str">
-        <v>2026-08-01T10:49:41.607Z</v>
+        <v>2026-08-08T07:13:21.357Z</v>
       </c>
       <c r="F217" t="str">
         <v>Success</v>
@@ -4753,7 +4753,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E218" t="str">
-        <v>2026-08-01T10:49:41.623Z</v>
+        <v>2026-08-08T07:13:21.373Z</v>
       </c>
       <c r="F218" t="str">
         <v>Success</v>
@@ -4773,7 +4773,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E219" t="str">
-        <v>2026-08-01T10:49:41.639Z</v>
+        <v>2026-08-08T07:13:21.389Z</v>
       </c>
       <c r="F219" t="str">
         <v>Success</v>
@@ -4793,7 +4793,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E220" t="str">
-        <v>2026-08-01T10:49:41.654Z</v>
+        <v>2026-08-08T07:13:21.404Z</v>
       </c>
       <c r="F220" t="str">
         <v>Success</v>
@@ -4813,7 +4813,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E221" t="str">
-        <v>2026-08-01T10:49:41.670Z</v>
+        <v>2026-08-08T07:13:21.420Z</v>
       </c>
       <c r="F221" t="str">
         <v>Success</v>
@@ -4830,10 +4830,10 @@
         <v>PASS</v>
       </c>
       <c r="D222" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E222" t="str">
-        <v>2026-08-01T10:49:41.685Z</v>
+        <v>2026-08-08T07:13:21.436Z</v>
       </c>
       <c r="F222" t="str">
         <v>Success</v>
@@ -4853,7 +4853,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E223" t="str">
-        <v>2026-08-01T10:49:41.701Z</v>
+        <v>2026-08-08T07:13:21.452Z</v>
       </c>
       <c r="F223" t="str">
         <v>Success</v>
@@ -4870,10 +4870,10 @@
         <v>PASS</v>
       </c>
       <c r="D224" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E224" t="str">
-        <v>2026-08-01T10:49:41.717Z</v>
+        <v>2026-08-08T07:13:21.467Z</v>
       </c>
       <c r="F224" t="str">
         <v>Success</v>
@@ -4890,10 +4890,10 @@
         <v>PASS</v>
       </c>
       <c r="D225" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E225" t="str">
-        <v>2026-08-01T10:49:41.733Z</v>
+        <v>2026-08-08T07:13:21.482Z</v>
       </c>
       <c r="F225" t="str">
         <v>Success</v>
@@ -4913,7 +4913,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E226" t="str">
-        <v>2026-08-01T10:49:41.749Z</v>
+        <v>2026-08-08T07:13:21.498Z</v>
       </c>
       <c r="F226" t="str">
         <v>Success</v>
@@ -4930,10 +4930,10 @@
         <v>PASS</v>
       </c>
       <c r="D227" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E227" t="str">
-        <v>2026-08-01T10:49:41.765Z</v>
+        <v>2026-08-08T07:13:21.513Z</v>
       </c>
       <c r="F227" t="str">
         <v>Success</v>
@@ -4953,7 +4953,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E228" t="str">
-        <v>2026-08-01T10:49:41.779Z</v>
+        <v>2026-08-08T07:13:21.528Z</v>
       </c>
       <c r="F228" t="str">
         <v>Success</v>
@@ -4970,10 +4970,10 @@
         <v>PASS</v>
       </c>
       <c r="D229" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E229" t="str">
-        <v>2026-08-01T10:49:41.794Z</v>
+        <v>2026-08-08T07:13:21.544Z</v>
       </c>
       <c r="F229" t="str">
         <v>Success</v>
@@ -4993,7 +4993,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E230" t="str">
-        <v>2026-08-01T10:49:41.809Z</v>
+        <v>2026-08-08T07:13:21.559Z</v>
       </c>
       <c r="F230" t="str">
         <v>Success</v>
@@ -5013,7 +5013,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E231" t="str">
-        <v>2026-08-01T10:49:41.825Z</v>
+        <v>2026-08-08T07:13:21.574Z</v>
       </c>
       <c r="F231" t="str">
         <v>Success</v>
@@ -5033,7 +5033,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E232" t="str">
-        <v>2026-08-01T10:49:41.841Z</v>
+        <v>2026-08-08T07:13:21.590Z</v>
       </c>
       <c r="F232" t="str">
         <v>Success</v>
@@ -5053,7 +5053,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E233" t="str">
-        <v>2026-08-01T10:49:41.855Z</v>
+        <v>2026-08-08T07:13:21.605Z</v>
       </c>
       <c r="F233" t="str">
         <v>Success</v>
@@ -5070,10 +5070,10 @@
         <v>PASS</v>
       </c>
       <c r="D234" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E234" t="str">
-        <v>2026-08-01T10:49:41.872Z</v>
+        <v>2026-08-08T07:13:21.620Z</v>
       </c>
       <c r="F234" t="str">
         <v>Success</v>
@@ -5093,7 +5093,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E235" t="str">
-        <v>2026-08-01T10:49:41.888Z</v>
+        <v>2026-08-08T07:13:21.636Z</v>
       </c>
       <c r="F235" t="str">
         <v>Success</v>
@@ -5110,10 +5110,10 @@
         <v>PASS</v>
       </c>
       <c r="D236" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E236" t="str">
-        <v>2026-08-01T10:49:41.903Z</v>
+        <v>2026-08-08T07:13:21.652Z</v>
       </c>
       <c r="F236" t="str">
         <v>Success</v>
@@ -5133,7 +5133,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E237" t="str">
-        <v>2026-08-01T10:49:41.919Z</v>
+        <v>2026-08-08T07:13:21.668Z</v>
       </c>
       <c r="F237" t="str">
         <v>Success</v>
@@ -5153,7 +5153,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E238" t="str">
-        <v>2026-08-01T10:49:41.935Z</v>
+        <v>2026-08-08T07:13:21.685Z</v>
       </c>
       <c r="F238" t="str">
         <v>Success</v>
@@ -5173,7 +5173,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E239" t="str">
-        <v>2026-08-01T10:49:41.950Z</v>
+        <v>2026-08-08T07:13:21.700Z</v>
       </c>
       <c r="F239" t="str">
         <v>Success</v>
@@ -5193,7 +5193,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E240" t="str">
-        <v>2026-08-01T10:49:41.966Z</v>
+        <v>2026-08-08T07:13:21.716Z</v>
       </c>
       <c r="F240" t="str">
         <v>Success</v>
@@ -5213,7 +5213,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E241" t="str">
-        <v>2026-08-01T10:49:41.982Z</v>
+        <v>2026-08-08T07:13:21.732Z</v>
       </c>
       <c r="F241" t="str">
         <v>Success</v>
@@ -5230,10 +5230,10 @@
         <v>PASS</v>
       </c>
       <c r="D242" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E242" t="str">
-        <v>2026-08-01T10:49:41.997Z</v>
+        <v>2026-08-08T07:13:21.748Z</v>
       </c>
       <c r="F242" t="str">
         <v>Success</v>
@@ -5253,7 +5253,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E243" t="str">
-        <v>2026-08-01T10:49:42.012Z</v>
+        <v>2026-08-08T07:13:21.763Z</v>
       </c>
       <c r="F243" t="str">
         <v>Success</v>
@@ -5270,10 +5270,10 @@
         <v>PASS</v>
       </c>
       <c r="D244" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E244" t="str">
-        <v>2026-08-01T10:49:42.028Z</v>
+        <v>2026-08-08T07:13:21.778Z</v>
       </c>
       <c r="F244" t="str">
         <v>Success</v>
@@ -5293,7 +5293,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E245" t="str">
-        <v>2026-08-01T10:49:42.044Z</v>
+        <v>2026-08-08T07:13:21.795Z</v>
       </c>
       <c r="F245" t="str">
         <v>Success</v>
@@ -5313,7 +5313,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E246" t="str">
-        <v>2026-08-01T10:49:42.059Z</v>
+        <v>2026-08-08T07:13:21.810Z</v>
       </c>
       <c r="F246" t="str">
         <v>Success</v>
@@ -5330,10 +5330,10 @@
         <v>PASS</v>
       </c>
       <c r="D247" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E247" t="str">
-        <v>2026-08-01T10:49:42.075Z</v>
+        <v>2026-08-08T07:13:21.825Z</v>
       </c>
       <c r="F247" t="str">
         <v>Success</v>
@@ -5350,10 +5350,10 @@
         <v>PASS</v>
       </c>
       <c r="D248" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E248" t="str">
-        <v>2026-08-01T10:49:42.090Z</v>
+        <v>2026-08-08T07:13:21.842Z</v>
       </c>
       <c r="F248" t="str">
         <v>Success</v>
@@ -5373,7 +5373,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E249" t="str">
-        <v>2026-08-01T10:49:42.105Z</v>
+        <v>2026-08-08T07:13:21.856Z</v>
       </c>
       <c r="F249" t="str">
         <v>Success</v>
@@ -5393,7 +5393,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E250" t="str">
-        <v>2026-08-01T10:49:42.121Z</v>
+        <v>2026-08-08T07:13:21.873Z</v>
       </c>
       <c r="F250" t="str">
         <v>Success</v>
@@ -5410,10 +5410,10 @@
         <v>PASS</v>
       </c>
       <c r="D251" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E251" t="str">
-        <v>2026-08-01T10:49:42.136Z</v>
+        <v>2026-08-08T07:13:21.889Z</v>
       </c>
       <c r="F251" t="str">
         <v>Success</v>
@@ -5430,10 +5430,10 @@
         <v>PASS</v>
       </c>
       <c r="D252" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E252" t="str">
-        <v>2026-08-01T10:49:42.152Z</v>
+        <v>2026-08-08T07:13:21.905Z</v>
       </c>
       <c r="F252" t="str">
         <v>Success</v>
@@ -5453,7 +5453,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E253" t="str">
-        <v>2026-08-01T10:49:42.167Z</v>
+        <v>2026-08-08T07:13:21.920Z</v>
       </c>
       <c r="F253" t="str">
         <v>Success</v>
@@ -5473,7 +5473,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E254" t="str">
-        <v>2026-08-01T10:49:42.183Z</v>
+        <v>2026-08-08T07:13:21.936Z</v>
       </c>
       <c r="F254" t="str">
         <v>Success</v>
@@ -5493,7 +5493,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E255" t="str">
-        <v>2026-08-01T10:49:42.199Z</v>
+        <v>2026-08-08T07:13:21.952Z</v>
       </c>
       <c r="F255" t="str">
         <v>Success</v>
@@ -5513,7 +5513,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E256" t="str">
-        <v>2026-08-01T10:49:42.214Z</v>
+        <v>2026-08-08T07:13:21.967Z</v>
       </c>
       <c r="F256" t="str">
         <v>Success</v>
@@ -5533,7 +5533,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E257" t="str">
-        <v>2026-08-01T10:49:42.230Z</v>
+        <v>2026-08-08T07:13:21.984Z</v>
       </c>
       <c r="F257" t="str">
         <v>Success</v>
@@ -5550,10 +5550,10 @@
         <v>PASS</v>
       </c>
       <c r="D258" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E258" t="str">
-        <v>2026-08-01T10:49:42.246Z</v>
+        <v>2026-08-08T07:13:21.999Z</v>
       </c>
       <c r="F258" t="str">
         <v>Success</v>
@@ -5570,10 +5570,10 @@
         <v>PASS</v>
       </c>
       <c r="D259" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E259" t="str">
-        <v>2026-08-01T10:49:42.262Z</v>
+        <v>2026-08-08T07:13:22.014Z</v>
       </c>
       <c r="F259" t="str">
         <v>Success</v>
@@ -5593,7 +5593,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E260" t="str">
-        <v>2026-08-01T10:49:42.277Z</v>
+        <v>2026-08-08T07:13:22.029Z</v>
       </c>
       <c r="F260" t="str">
         <v>Success</v>
@@ -5613,7 +5613,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E261" t="str">
-        <v>2026-08-01T10:49:42.293Z</v>
+        <v>2026-08-08T07:13:22.045Z</v>
       </c>
       <c r="F261" t="str">
         <v>Success</v>
@@ -5633,7 +5633,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E262" t="str">
-        <v>2026-08-01T10:49:42.308Z</v>
+        <v>2026-08-08T07:13:22.061Z</v>
       </c>
       <c r="F262" t="str">
         <v>Success</v>
@@ -5653,7 +5653,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E263" t="str">
-        <v>2026-08-01T10:49:42.324Z</v>
+        <v>2026-08-08T07:13:22.077Z</v>
       </c>
       <c r="F263" t="str">
         <v>Success</v>
@@ -5673,7 +5673,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E264" t="str">
-        <v>2026-08-01T10:49:42.339Z</v>
+        <v>2026-08-08T07:13:22.092Z</v>
       </c>
       <c r="F264" t="str">
         <v>Success</v>
@@ -5693,7 +5693,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E265" t="str">
-        <v>2026-08-01T10:49:42.355Z</v>
+        <v>2026-08-08T07:13:22.108Z</v>
       </c>
       <c r="F265" t="str">
         <v>Success</v>
@@ -5710,10 +5710,10 @@
         <v>PASS</v>
       </c>
       <c r="D266" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E266" t="str">
-        <v>2026-08-01T10:49:42.372Z</v>
+        <v>2026-08-08T07:13:22.123Z</v>
       </c>
       <c r="F266" t="str">
         <v>Success</v>
@@ -5733,7 +5733,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E267" t="str">
-        <v>2026-08-01T10:49:42.386Z</v>
+        <v>2026-08-08T07:13:22.138Z</v>
       </c>
       <c r="F267" t="str">
         <v>Success</v>
@@ -5753,7 +5753,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E268" t="str">
-        <v>2026-08-01T10:49:42.402Z</v>
+        <v>2026-08-08T07:13:22.154Z</v>
       </c>
       <c r="F268" t="str">
         <v>Success</v>
@@ -5773,7 +5773,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E269" t="str">
-        <v>2026-08-01T10:49:42.417Z</v>
+        <v>2026-08-08T07:13:22.169Z</v>
       </c>
       <c r="F269" t="str">
         <v>Success</v>
@@ -5793,7 +5793,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E270" t="str">
-        <v>2026-08-01T10:49:42.433Z</v>
+        <v>2026-08-08T07:13:22.185Z</v>
       </c>
       <c r="F270" t="str">
         <v>Success</v>
@@ -5810,10 +5810,10 @@
         <v>PASS</v>
       </c>
       <c r="D271" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E271" t="str">
-        <v>2026-08-01T10:49:42.449Z</v>
+        <v>2026-08-08T07:13:22.200Z</v>
       </c>
       <c r="F271" t="str">
         <v>Success</v>
@@ -5833,7 +5833,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E272" t="str">
-        <v>2026-08-01T10:49:42.464Z</v>
+        <v>2026-08-08T07:13:22.216Z</v>
       </c>
       <c r="F272" t="str">
         <v>Success</v>
@@ -5850,10 +5850,10 @@
         <v>PASS</v>
       </c>
       <c r="D273" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E273" t="str">
-        <v>2026-08-01T10:49:42.480Z</v>
+        <v>2026-08-08T07:13:22.231Z</v>
       </c>
       <c r="F273" t="str">
         <v>Success</v>
@@ -5873,7 +5873,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E274" t="str">
-        <v>2026-08-01T10:49:42.495Z</v>
+        <v>2026-08-08T07:13:22.247Z</v>
       </c>
       <c r="F274" t="str">
         <v>Success</v>
@@ -5890,10 +5890,10 @@
         <v>PASS</v>
       </c>
       <c r="D275" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E275" t="str">
-        <v>2026-08-01T10:49:42.511Z</v>
+        <v>2026-08-08T07:13:22.262Z</v>
       </c>
       <c r="F275" t="str">
         <v>Success</v>
@@ -5910,10 +5910,10 @@
         <v>PASS</v>
       </c>
       <c r="D276" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E276" t="str">
-        <v>2026-08-01T10:49:42.525Z</v>
+        <v>2026-08-08T07:13:22.278Z</v>
       </c>
       <c r="F276" t="str">
         <v>Success</v>
@@ -5933,7 +5933,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E277" t="str">
-        <v>2026-08-01T10:49:42.540Z</v>
+        <v>2026-08-08T07:13:22.294Z</v>
       </c>
       <c r="F277" t="str">
         <v>Success</v>
@@ -5953,7 +5953,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E278" t="str">
-        <v>2026-08-01T10:49:42.555Z</v>
+        <v>2026-08-08T07:13:22.309Z</v>
       </c>
       <c r="F278" t="str">
         <v>Success</v>
@@ -5970,10 +5970,10 @@
         <v>PASS</v>
       </c>
       <c r="D279" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E279" t="str">
-        <v>2026-08-01T10:49:42.571Z</v>
+        <v>2026-08-08T07:13:22.325Z</v>
       </c>
       <c r="F279" t="str">
         <v>Success</v>
@@ -5990,10 +5990,10 @@
         <v>PASS</v>
       </c>
       <c r="D280" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E280" t="str">
-        <v>2026-08-01T10:49:42.587Z</v>
+        <v>2026-08-08T07:13:22.341Z</v>
       </c>
       <c r="F280" t="str">
         <v>Success</v>
@@ -6010,10 +6010,10 @@
         <v>PASS</v>
       </c>
       <c r="D281" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E281" t="str">
-        <v>2026-08-01T10:49:42.603Z</v>
+        <v>2026-08-08T07:13:22.356Z</v>
       </c>
       <c r="F281" t="str">
         <v>Success</v>
@@ -6033,7 +6033,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E282" t="str">
-        <v>2026-08-01T10:49:42.618Z</v>
+        <v>2026-08-08T07:13:22.371Z</v>
       </c>
       <c r="F282" t="str">
         <v>Success</v>
@@ -6050,10 +6050,10 @@
         <v>PASS</v>
       </c>
       <c r="D283" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E283" t="str">
-        <v>2026-08-01T10:49:42.633Z</v>
+        <v>2026-08-08T07:13:22.387Z</v>
       </c>
       <c r="F283" t="str">
         <v>Success</v>
@@ -6073,7 +6073,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E284" t="str">
-        <v>2026-08-01T10:49:42.649Z</v>
+        <v>2026-08-08T07:13:22.403Z</v>
       </c>
       <c r="F284" t="str">
         <v>Success</v>
@@ -6090,10 +6090,10 @@
         <v>PASS</v>
       </c>
       <c r="D285" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E285" t="str">
-        <v>2026-08-01T10:49:42.664Z</v>
+        <v>2026-08-08T07:13:22.419Z</v>
       </c>
       <c r="F285" t="str">
         <v>Success</v>
@@ -6113,7 +6113,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E286" t="str">
-        <v>2026-08-01T10:49:42.680Z</v>
+        <v>2026-08-08T07:13:22.435Z</v>
       </c>
       <c r="F286" t="str">
         <v>Success</v>
@@ -6130,10 +6130,10 @@
         <v>PASS</v>
       </c>
       <c r="D287" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E287" t="str">
-        <v>2026-08-01T10:49:42.696Z</v>
+        <v>2026-08-08T07:13:22.450Z</v>
       </c>
       <c r="F287" t="str">
         <v>Success</v>
@@ -6150,10 +6150,10 @@
         <v>PASS</v>
       </c>
       <c r="D288" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E288" t="str">
-        <v>2026-08-01T10:49:42.711Z</v>
+        <v>2026-08-08T07:13:22.466Z</v>
       </c>
       <c r="F288" t="str">
         <v>Success</v>
@@ -6173,7 +6173,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E289" t="str">
-        <v>2026-08-01T10:49:42.727Z</v>
+        <v>2026-08-08T07:13:22.482Z</v>
       </c>
       <c r="F289" t="str">
         <v>Success</v>
@@ -6193,7 +6193,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E290" t="str">
-        <v>2026-08-01T10:49:42.742Z</v>
+        <v>2026-08-08T07:13:22.497Z</v>
       </c>
       <c r="F290" t="str">
         <v>Success</v>
@@ -6210,10 +6210,10 @@
         <v>PASS</v>
       </c>
       <c r="D291" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E291" t="str">
-        <v>2026-08-01T10:49:42.758Z</v>
+        <v>2026-08-08T07:13:22.513Z</v>
       </c>
       <c r="F291" t="str">
         <v>Success</v>
@@ -6233,7 +6233,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E292" t="str">
-        <v>2026-08-01T10:49:42.774Z</v>
+        <v>2026-08-08T07:13:22.528Z</v>
       </c>
       <c r="F292" t="str">
         <v>Success</v>
@@ -6250,10 +6250,10 @@
         <v>PASS</v>
       </c>
       <c r="D293" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E293" t="str">
-        <v>2026-08-01T10:49:42.789Z</v>
+        <v>2026-08-08T07:13:22.544Z</v>
       </c>
       <c r="F293" t="str">
         <v>Success</v>
@@ -6273,7 +6273,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E294" t="str">
-        <v>2026-08-01T10:49:42.805Z</v>
+        <v>2026-08-08T07:13:22.560Z</v>
       </c>
       <c r="F294" t="str">
         <v>Success</v>
@@ -6293,7 +6293,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E295" t="str">
-        <v>2026-08-01T10:49:42.820Z</v>
+        <v>2026-08-08T07:13:22.575Z</v>
       </c>
       <c r="F295" t="str">
         <v>Success</v>
@@ -6310,10 +6310,10 @@
         <v>PASS</v>
       </c>
       <c r="D296" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E296" t="str">
-        <v>2026-08-01T10:49:42.835Z</v>
+        <v>2026-08-08T07:13:22.591Z</v>
       </c>
       <c r="F296" t="str">
         <v>Success</v>
@@ -6330,10 +6330,10 @@
         <v>PASS</v>
       </c>
       <c r="D297" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E297" t="str">
-        <v>2026-08-01T10:49:42.851Z</v>
+        <v>2026-08-08T07:13:22.606Z</v>
       </c>
       <c r="F297" t="str">
         <v>Success</v>
@@ -6353,7 +6353,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E298" t="str">
-        <v>2026-08-01T10:49:42.867Z</v>
+        <v>2026-08-08T07:13:22.622Z</v>
       </c>
       <c r="F298" t="str">
         <v>Success</v>
@@ -6370,10 +6370,10 @@
         <v>PASS</v>
       </c>
       <c r="D299" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E299" t="str">
-        <v>2026-08-01T10:49:42.883Z</v>
+        <v>2026-08-08T07:13:22.637Z</v>
       </c>
       <c r="F299" t="str">
         <v>Success</v>
@@ -6390,10 +6390,10 @@
         <v>PASS</v>
       </c>
       <c r="D300" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E300" t="str">
-        <v>2026-08-01T10:49:42.898Z</v>
+        <v>2026-08-08T07:13:22.654Z</v>
       </c>
       <c r="F300" t="str">
         <v>Success</v>
@@ -6413,7 +6413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E301" t="str">
-        <v>2026-08-01T10:49:42.913Z</v>
+        <v>2026-08-08T07:13:22.669Z</v>
       </c>
       <c r="F301" t="str">
         <v>Success</v>
@@ -6433,7 +6433,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E302" t="str">
-        <v>2026-08-01T10:49:42.928Z</v>
+        <v>2026-08-08T07:13:22.684Z</v>
       </c>
       <c r="F302" t="str">
         <v>Success</v>
@@ -6453,7 +6453,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E303" t="str">
-        <v>2026-08-01T10:49:42.944Z</v>
+        <v>2026-08-08T07:13:22.700Z</v>
       </c>
       <c r="F303" t="str">
         <v>Success</v>
@@ -6470,10 +6470,10 @@
         <v>PASS</v>
       </c>
       <c r="D304" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E304" t="str">
-        <v>2026-08-01T10:49:42.960Z</v>
+        <v>2026-08-08T07:13:22.715Z</v>
       </c>
       <c r="F304" t="str">
         <v>Success</v>
@@ -6490,10 +6490,10 @@
         <v>PASS</v>
       </c>
       <c r="D305" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E305" t="str">
-        <v>2026-08-01T10:49:42.975Z</v>
+        <v>2026-08-08T07:13:22.732Z</v>
       </c>
       <c r="F305" t="str">
         <v>Success</v>
@@ -6510,10 +6510,10 @@
         <v>PASS</v>
       </c>
       <c r="D306" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E306" t="str">
-        <v>2026-08-01T10:49:42.991Z</v>
+        <v>2026-08-08T07:13:22.747Z</v>
       </c>
       <c r="F306" t="str">
         <v>Success</v>
@@ -6533,7 +6533,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E307" t="str">
-        <v>2026-08-01T10:49:43.007Z</v>
+        <v>2026-08-08T07:13:22.763Z</v>
       </c>
       <c r="F307" t="str">
         <v>Success</v>
@@ -6550,10 +6550,10 @@
         <v>PASS</v>
       </c>
       <c r="D308" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E308" t="str">
-        <v>2026-08-01T10:49:43.023Z</v>
+        <v>2026-08-08T07:13:22.778Z</v>
       </c>
       <c r="F308" t="str">
         <v>Success</v>
@@ -6573,7 +6573,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E309" t="str">
-        <v>2026-08-01T10:49:43.039Z</v>
+        <v>2026-08-08T07:13:22.794Z</v>
       </c>
       <c r="F309" t="str">
         <v>Success</v>
@@ -6593,7 +6593,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E310" t="str">
-        <v>2026-08-01T10:49:43.055Z</v>
+        <v>2026-08-08T07:13:22.809Z</v>
       </c>
       <c r="F310" t="str">
         <v>Success</v>
@@ -6610,10 +6610,10 @@
         <v>PASS</v>
       </c>
       <c r="D311" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E311" t="str">
-        <v>2026-08-01T10:49:43.070Z</v>
+        <v>2026-08-08T07:13:22.825Z</v>
       </c>
       <c r="F311" t="str">
         <v>Success</v>
@@ -6630,10 +6630,10 @@
         <v>PASS</v>
       </c>
       <c r="D312" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E312" t="str">
-        <v>2026-08-01T10:49:43.086Z</v>
+        <v>2026-08-08T07:13:22.840Z</v>
       </c>
       <c r="F312" t="str">
         <v>Success</v>
@@ -6653,7 +6653,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E313" t="str">
-        <v>2026-08-01T10:49:43.101Z</v>
+        <v>2026-08-08T07:13:22.855Z</v>
       </c>
       <c r="F313" t="str">
         <v>Success</v>
@@ -6673,7 +6673,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E314" t="str">
-        <v>2026-08-01T10:49:43.117Z</v>
+        <v>2026-08-08T07:13:22.872Z</v>
       </c>
       <c r="F314" t="str">
         <v>Success</v>
@@ -6690,10 +6690,10 @@
         <v>PASS</v>
       </c>
       <c r="D315" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E315" t="str">
-        <v>2026-08-01T10:49:43.134Z</v>
+        <v>2026-08-08T07:13:22.887Z</v>
       </c>
       <c r="F315" t="str">
         <v>Success</v>
@@ -6710,10 +6710,10 @@
         <v>PASS</v>
       </c>
       <c r="D316" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E316" t="str">
-        <v>2026-08-01T10:49:43.150Z</v>
+        <v>2026-08-08T07:13:22.903Z</v>
       </c>
       <c r="F316" t="str">
         <v>Success</v>
@@ -6730,10 +6730,10 @@
         <v>PASS</v>
       </c>
       <c r="D317" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E317" t="str">
-        <v>2026-08-01T10:49:43.164Z</v>
+        <v>2026-08-08T07:13:22.919Z</v>
       </c>
       <c r="F317" t="str">
         <v>Success</v>
@@ -6753,7 +6753,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E318" t="str">
-        <v>2026-08-01T10:49:43.180Z</v>
+        <v>2026-08-08T07:13:22.935Z</v>
       </c>
       <c r="F318" t="str">
         <v>Success</v>
@@ -6770,10 +6770,10 @@
         <v>PASS</v>
       </c>
       <c r="D319" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E319" t="str">
-        <v>2026-08-01T10:49:43.196Z</v>
+        <v>2026-08-08T07:13:22.950Z</v>
       </c>
       <c r="F319" t="str">
         <v>Success</v>
@@ -6790,10 +6790,10 @@
         <v>PASS</v>
       </c>
       <c r="D320" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E320" t="str">
-        <v>2026-08-01T10:49:43.211Z</v>
+        <v>2026-08-08T07:13:22.966Z</v>
       </c>
       <c r="F320" t="str">
         <v>Success</v>
@@ -6813,7 +6813,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E321" t="str">
-        <v>2026-08-01T10:49:43.226Z</v>
+        <v>2026-08-08T07:13:22.981Z</v>
       </c>
       <c r="F321" t="str">
         <v>Success</v>
@@ -6830,10 +6830,10 @@
         <v>PASS</v>
       </c>
       <c r="D322" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E322" t="str">
-        <v>2026-08-01T10:49:43.242Z</v>
+        <v>2026-08-08T07:13:22.997Z</v>
       </c>
       <c r="F322" t="str">
         <v>Success</v>
@@ -6850,10 +6850,10 @@
         <v>PASS</v>
       </c>
       <c r="D323" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E323" t="str">
-        <v>2026-08-01T10:49:43.257Z</v>
+        <v>2026-08-08T07:13:23.013Z</v>
       </c>
       <c r="F323" t="str">
         <v>Success</v>
@@ -6870,10 +6870,10 @@
         <v>PASS</v>
       </c>
       <c r="D324" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E324" t="str">
-        <v>2026-08-01T10:49:43.273Z</v>
+        <v>2026-08-08T07:13:23.028Z</v>
       </c>
       <c r="F324" t="str">
         <v>Success</v>
@@ -6890,10 +6890,10 @@
         <v>PASS</v>
       </c>
       <c r="D325" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E325" t="str">
-        <v>2026-08-01T10:49:43.289Z</v>
+        <v>2026-08-08T07:13:23.044Z</v>
       </c>
       <c r="F325" t="str">
         <v>Success</v>
@@ -6913,7 +6913,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E326" t="str">
-        <v>2026-08-01T10:49:43.305Z</v>
+        <v>2026-08-08T07:13:23.060Z</v>
       </c>
       <c r="F326" t="str">
         <v>Success</v>
@@ -6933,7 +6933,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E327" t="str">
-        <v>2026-08-01T10:49:43.320Z</v>
+        <v>2026-08-08T07:13:23.075Z</v>
       </c>
       <c r="F327" t="str">
         <v>Success</v>
@@ -6950,10 +6950,10 @@
         <v>PASS</v>
       </c>
       <c r="D328" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E328" t="str">
-        <v>2026-08-01T10:49:43.336Z</v>
+        <v>2026-08-08T07:13:23.090Z</v>
       </c>
       <c r="F328" t="str">
         <v>Success</v>
@@ -6973,7 +6973,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E329" t="str">
-        <v>2026-08-01T10:49:43.352Z</v>
+        <v>2026-08-08T07:13:23.106Z</v>
       </c>
       <c r="F329" t="str">
         <v>Success</v>
@@ -6990,10 +6990,10 @@
         <v>PASS</v>
       </c>
       <c r="D330" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E330" t="str">
-        <v>2026-08-01T10:49:43.368Z</v>
+        <v>2026-08-08T07:13:23.121Z</v>
       </c>
       <c r="F330" t="str">
         <v>Success</v>
@@ -7013,7 +7013,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E331" t="str">
-        <v>2026-08-01T10:49:43.383Z</v>
+        <v>2026-08-08T07:13:23.136Z</v>
       </c>
       <c r="F331" t="str">
         <v>Success</v>
@@ -7030,10 +7030,10 @@
         <v>PASS</v>
       </c>
       <c r="D332" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E332" t="str">
-        <v>2026-08-01T10:49:43.399Z</v>
+        <v>2026-08-08T07:13:23.152Z</v>
       </c>
       <c r="F332" t="str">
         <v>Success</v>
@@ -7050,10 +7050,10 @@
         <v>PASS</v>
       </c>
       <c r="D333" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E333" t="str">
-        <v>2026-08-01T10:49:43.414Z</v>
+        <v>2026-08-08T07:13:23.168Z</v>
       </c>
       <c r="F333" t="str">
         <v>Success</v>
@@ -7070,10 +7070,10 @@
         <v>PASS</v>
       </c>
       <c r="D334" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E334" t="str">
-        <v>2026-08-01T10:49:43.430Z</v>
+        <v>2026-08-08T07:13:23.183Z</v>
       </c>
       <c r="F334" t="str">
         <v>Success</v>
@@ -7093,7 +7093,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E335" t="str">
-        <v>2026-08-01T10:49:43.446Z</v>
+        <v>2026-08-08T07:13:23.199Z</v>
       </c>
       <c r="F335" t="str">
         <v>Success</v>
@@ -7110,10 +7110,10 @@
         <v>PASS</v>
       </c>
       <c r="D336" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E336" t="str">
-        <v>2026-08-01T10:49:43.462Z</v>
+        <v>2026-08-08T07:13:23.214Z</v>
       </c>
       <c r="F336" t="str">
         <v>Success</v>
@@ -7130,10 +7130,10 @@
         <v>PASS</v>
       </c>
       <c r="D337" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E337" t="str">
-        <v>2026-08-01T10:49:43.477Z</v>
+        <v>2026-08-08T07:13:23.230Z</v>
       </c>
       <c r="F337" t="str">
         <v>Success</v>
@@ -7150,10 +7150,10 @@
         <v>PASS</v>
       </c>
       <c r="D338" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E338" t="str">
-        <v>2026-08-01T10:49:43.492Z</v>
+        <v>2026-08-08T07:13:23.247Z</v>
       </c>
       <c r="F338" t="str">
         <v>Success</v>
@@ -7173,7 +7173,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E339" t="str">
-        <v>2026-08-01T10:49:43.508Z</v>
+        <v>2026-08-08T07:13:23.265Z</v>
       </c>
       <c r="F339" t="str">
         <v>Success</v>
@@ -7193,7 +7193,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E340" t="str">
-        <v>2026-08-01T10:49:43.523Z</v>
+        <v>2026-08-08T07:13:23.278Z</v>
       </c>
       <c r="F340" t="str">
         <v>Success</v>
@@ -7210,10 +7210,10 @@
         <v>PASS</v>
       </c>
       <c r="D341" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E341" t="str">
-        <v>2026-08-01T10:49:43.539Z</v>
+        <v>2026-08-08T07:13:23.293Z</v>
       </c>
       <c r="F341" t="str">
         <v>Success</v>
@@ -7230,10 +7230,10 @@
         <v>PASS</v>
       </c>
       <c r="D342" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E342" t="str">
-        <v>2026-08-01T10:49:43.555Z</v>
+        <v>2026-08-08T07:13:23.308Z</v>
       </c>
       <c r="F342" t="str">
         <v>Success</v>
@@ -7253,7 +7253,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E343" t="str">
-        <v>2026-08-01T10:49:43.571Z</v>
+        <v>2026-08-08T07:13:23.324Z</v>
       </c>
       <c r="F343" t="str">
         <v>Success</v>
@@ -7273,7 +7273,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E344" t="str">
-        <v>2026-08-01T10:49:43.587Z</v>
+        <v>2026-08-08T07:13:23.343Z</v>
       </c>
       <c r="F344" t="str">
         <v>Success</v>
@@ -7293,7 +7293,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E345" t="str">
-        <v>2026-08-01T10:49:43.602Z</v>
+        <v>2026-08-08T07:13:23.356Z</v>
       </c>
       <c r="F345" t="str">
         <v>Success</v>
@@ -7310,10 +7310,10 @@
         <v>PASS</v>
       </c>
       <c r="D346" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E346" t="str">
-        <v>2026-08-01T10:49:43.618Z</v>
+        <v>2026-08-08T07:13:23.371Z</v>
       </c>
       <c r="F346" t="str">
         <v>Success</v>
@@ -7330,10 +7330,10 @@
         <v>PASS</v>
       </c>
       <c r="D347" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E347" t="str">
-        <v>2026-08-01T10:49:43.633Z</v>
+        <v>2026-08-08T07:13:23.387Z</v>
       </c>
       <c r="F347" t="str">
         <v>Success</v>
@@ -7350,10 +7350,10 @@
         <v>PASS</v>
       </c>
       <c r="D348" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E348" t="str">
-        <v>2026-08-01T10:49:43.649Z</v>
+        <v>2026-08-08T07:13:23.401Z</v>
       </c>
       <c r="F348" t="str">
         <v>Success</v>
@@ -7373,7 +7373,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E349" t="str">
-        <v>2026-08-01T10:49:43.665Z</v>
+        <v>2026-08-08T07:13:23.418Z</v>
       </c>
       <c r="F349" t="str">
         <v>Success</v>
@@ -7393,7 +7393,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E350" t="str">
-        <v>2026-08-01T10:49:43.681Z</v>
+        <v>2026-08-08T07:13:23.434Z</v>
       </c>
       <c r="F350" t="str">
         <v>Success</v>
@@ -7413,7 +7413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E351" t="str">
-        <v>2026-08-01T10:49:43.696Z</v>
+        <v>2026-08-08T07:13:23.449Z</v>
       </c>
       <c r="F351" t="str">
         <v>Success</v>
@@ -7433,7 +7433,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E352" t="str">
-        <v>2026-08-01T10:49:43.712Z</v>
+        <v>2026-08-08T07:13:23.465Z</v>
       </c>
       <c r="F352" t="str">
         <v>Success</v>
@@ -7450,10 +7450,10 @@
         <v>PASS</v>
       </c>
       <c r="D353" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E353" t="str">
-        <v>2026-08-01T10:49:43.728Z</v>
+        <v>2026-08-08T07:13:23.479Z</v>
       </c>
       <c r="F353" t="str">
         <v>Success</v>
@@ -7470,10 +7470,10 @@
         <v>PASS</v>
       </c>
       <c r="D354" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E354" t="str">
-        <v>2026-08-01T10:49:43.743Z</v>
+        <v>2026-08-08T07:13:23.495Z</v>
       </c>
       <c r="F354" t="str">
         <v>Success</v>
@@ -7493,7 +7493,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E355" t="str">
-        <v>2026-08-01T10:49:43.759Z</v>
+        <v>2026-08-08T07:13:23.511Z</v>
       </c>
       <c r="F355" t="str">
         <v>Success</v>
@@ -7510,10 +7510,10 @@
         <v>PASS</v>
       </c>
       <c r="D356" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E356" t="str">
-        <v>2026-08-01T10:49:43.774Z</v>
+        <v>2026-08-08T07:13:23.527Z</v>
       </c>
       <c r="F356" t="str">
         <v>Success</v>
@@ -7533,7 +7533,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E357" t="str">
-        <v>2026-08-01T10:49:43.790Z</v>
+        <v>2026-08-08T07:13:23.543Z</v>
       </c>
       <c r="F357" t="str">
         <v>Success</v>
@@ -7550,10 +7550,10 @@
         <v>PASS</v>
       </c>
       <c r="D358" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E358" t="str">
-        <v>2026-08-01T10:49:43.806Z</v>
+        <v>2026-08-08T07:13:23.558Z</v>
       </c>
       <c r="F358" t="str">
         <v>Success</v>
@@ -7573,7 +7573,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E359" t="str">
-        <v>2026-08-01T10:49:43.821Z</v>
+        <v>2026-08-08T07:13:23.573Z</v>
       </c>
       <c r="F359" t="str">
         <v>Success</v>
@@ -7593,7 +7593,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E360" t="str">
-        <v>2026-08-01T10:49:43.837Z</v>
+        <v>2026-08-08T07:13:23.589Z</v>
       </c>
       <c r="F360" t="str">
         <v>Success</v>
@@ -7610,10 +7610,10 @@
         <v>PASS</v>
       </c>
       <c r="D361" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E361" t="str">
-        <v>2026-08-01T10:49:43.852Z</v>
+        <v>2026-08-08T07:13:23.605Z</v>
       </c>
       <c r="F361" t="str">
         <v>Success</v>
@@ -7633,7 +7633,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E362" t="str">
-        <v>2026-08-01T10:49:43.868Z</v>
+        <v>2026-08-08T07:13:23.621Z</v>
       </c>
       <c r="F362" t="str">
         <v>Success</v>
@@ -7653,7 +7653,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E363" t="str">
-        <v>2026-08-01T10:49:43.884Z</v>
+        <v>2026-08-08T07:13:23.637Z</v>
       </c>
       <c r="F363" t="str">
         <v>Success</v>
@@ -7673,7 +7673,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E364" t="str">
-        <v>2026-08-01T10:49:43.899Z</v>
+        <v>2026-08-08T07:13:23.652Z</v>
       </c>
       <c r="F364" t="str">
         <v>Success</v>
@@ -7690,10 +7690,10 @@
         <v>PASS</v>
       </c>
       <c r="D365" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E365" t="str">
-        <v>2026-08-01T10:49:43.915Z</v>
+        <v>2026-08-08T07:13:23.667Z</v>
       </c>
       <c r="F365" t="str">
         <v>Success</v>
@@ -7710,10 +7710,10 @@
         <v>PASS</v>
       </c>
       <c r="D366" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E366" t="str">
-        <v>2026-08-01T10:49:43.931Z</v>
+        <v>2026-08-08T07:13:23.682Z</v>
       </c>
       <c r="F366" t="str">
         <v>Success</v>
@@ -7733,7 +7733,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E367" t="str">
-        <v>2026-08-01T10:49:43.947Z</v>
+        <v>2026-08-08T07:13:23.698Z</v>
       </c>
       <c r="F367" t="str">
         <v>Success</v>
@@ -7750,10 +7750,10 @@
         <v>PASS</v>
       </c>
       <c r="D368" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E368" t="str">
-        <v>2026-08-01T10:49:43.962Z</v>
+        <v>2026-08-08T07:13:23.714Z</v>
       </c>
       <c r="F368" t="str">
         <v>Success</v>
@@ -7773,7 +7773,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E369" t="str">
-        <v>2026-08-01T10:49:43.977Z</v>
+        <v>2026-08-08T07:13:23.729Z</v>
       </c>
       <c r="F369" t="str">
         <v>Success</v>
@@ -7793,7 +7793,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E370" t="str">
-        <v>2026-08-01T10:49:43.993Z</v>
+        <v>2026-08-08T07:13:23.746Z</v>
       </c>
       <c r="F370" t="str">
         <v>Success</v>
@@ -7810,10 +7810,10 @@
         <v>PASS</v>
       </c>
       <c r="D371" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E371" t="str">
-        <v>2026-08-01T10:49:44.008Z</v>
+        <v>2026-08-08T07:13:23.763Z</v>
       </c>
       <c r="F371" t="str">
         <v>Success</v>
@@ -7833,7 +7833,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E372" t="str">
-        <v>2026-08-01T10:49:44.023Z</v>
+        <v>2026-08-08T07:13:23.777Z</v>
       </c>
       <c r="F372" t="str">
         <v>Success</v>
@@ -7853,7 +7853,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E373" t="str">
-        <v>2026-08-01T10:49:44.039Z</v>
+        <v>2026-08-08T07:13:23.793Z</v>
       </c>
       <c r="F373" t="str">
         <v>Success</v>
@@ -7870,10 +7870,10 @@
         <v>PASS</v>
       </c>
       <c r="D374" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E374" t="str">
-        <v>2026-08-01T10:49:44.054Z</v>
+        <v>2026-08-08T07:13:23.809Z</v>
       </c>
       <c r="F374" t="str">
         <v>Success</v>
@@ -7890,10 +7890,10 @@
         <v>PASS</v>
       </c>
       <c r="D375" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E375" t="str">
-        <v>2026-08-01T10:49:44.070Z</v>
+        <v>2026-08-08T07:13:23.824Z</v>
       </c>
       <c r="F375" t="str">
         <v>Success</v>
@@ -7913,7 +7913,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E376" t="str">
-        <v>2026-08-01T10:49:44.085Z</v>
+        <v>2026-08-08T07:13:23.839Z</v>
       </c>
       <c r="F376" t="str">
         <v>Success</v>
@@ -7930,10 +7930,10 @@
         <v>PASS</v>
       </c>
       <c r="D377" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E377" t="str">
-        <v>2026-08-01T10:49:44.101Z</v>
+        <v>2026-08-08T07:13:23.854Z</v>
       </c>
       <c r="F377" t="str">
         <v>Success</v>
@@ -7953,7 +7953,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E378" t="str">
-        <v>2026-08-01T10:49:44.116Z</v>
+        <v>2026-08-08T07:13:23.870Z</v>
       </c>
       <c r="F378" t="str">
         <v>Success</v>
@@ -7973,7 +7973,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E379" t="str">
-        <v>2026-08-01T10:49:44.132Z</v>
+        <v>2026-08-08T07:13:23.886Z</v>
       </c>
       <c r="F379" t="str">
         <v>Success</v>
@@ -7993,7 +7993,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E380" t="str">
-        <v>2026-08-01T10:49:44.147Z</v>
+        <v>2026-08-08T07:13:23.900Z</v>
       </c>
       <c r="F380" t="str">
         <v>Success</v>
@@ -8010,10 +8010,10 @@
         <v>PASS</v>
       </c>
       <c r="D381" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E381" t="str">
-        <v>2026-08-01T10:49:44.163Z</v>
+        <v>2026-08-08T07:13:23.915Z</v>
       </c>
       <c r="F381" t="str">
         <v>Success</v>
@@ -8030,10 +8030,10 @@
         <v>PASS</v>
       </c>
       <c r="D382" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E382" t="str">
-        <v>2026-08-01T10:49:44.178Z</v>
+        <v>2026-08-08T07:13:23.932Z</v>
       </c>
       <c r="F382" t="str">
         <v>Success</v>
@@ -8050,10 +8050,10 @@
         <v>PASS</v>
       </c>
       <c r="D383" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E383" t="str">
-        <v>2026-08-01T10:49:44.194Z</v>
+        <v>2026-08-08T07:13:23.947Z</v>
       </c>
       <c r="F383" t="str">
         <v>Success</v>
@@ -8070,10 +8070,10 @@
         <v>PASS</v>
       </c>
       <c r="D384" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E384" t="str">
-        <v>2026-08-01T10:49:44.210Z</v>
+        <v>2026-08-08T07:13:23.963Z</v>
       </c>
       <c r="F384" t="str">
         <v>Success</v>
@@ -8090,10 +8090,10 @@
         <v>PASS</v>
       </c>
       <c r="D385" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E385" t="str">
-        <v>2026-08-01T10:49:44.225Z</v>
+        <v>2026-08-08T07:13:23.979Z</v>
       </c>
       <c r="F385" t="str">
         <v>Success</v>
@@ -8110,10 +8110,10 @@
         <v>PASS</v>
       </c>
       <c r="D386" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E386" t="str">
-        <v>2026-08-01T10:49:44.240Z</v>
+        <v>2026-08-08T07:13:23.995Z</v>
       </c>
       <c r="F386" t="str">
         <v>Success</v>
@@ -8130,10 +8130,10 @@
         <v>PASS</v>
       </c>
       <c r="D387" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E387" t="str">
-        <v>2026-08-01T10:49:44.255Z</v>
+        <v>2026-08-08T07:13:24.011Z</v>
       </c>
       <c r="F387" t="str">
         <v>Success</v>
@@ -8150,10 +8150,10 @@
         <v>PASS</v>
       </c>
       <c r="D388" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E388" t="str">
-        <v>2026-08-01T10:49:44.271Z</v>
+        <v>2026-08-08T07:13:24.026Z</v>
       </c>
       <c r="F388" t="str">
         <v>Success</v>
@@ -8170,10 +8170,10 @@
         <v>PASS</v>
       </c>
       <c r="D389" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E389" t="str">
-        <v>2026-08-01T10:49:44.286Z</v>
+        <v>2026-08-08T07:13:24.043Z</v>
       </c>
       <c r="F389" t="str">
         <v>Success</v>
@@ -8190,10 +8190,10 @@
         <v>PASS</v>
       </c>
       <c r="D390" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E390" t="str">
-        <v>2026-08-01T10:49:44.302Z</v>
+        <v>2026-08-08T07:13:24.059Z</v>
       </c>
       <c r="F390" t="str">
         <v>Success</v>
@@ -8210,10 +8210,10 @@
         <v>PASS</v>
       </c>
       <c r="D391" t="str">
-        <v>0.02 sec</v>
+        <v>0.01 sec</v>
       </c>
       <c r="E391" t="str">
-        <v>2026-08-01T10:49:44.318Z</v>
+        <v>2026-08-08T07:13:24.073Z</v>
       </c>
       <c r="F391" t="str">
         <v>Success</v>
@@ -8233,7 +8233,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E392" t="str">
-        <v>2026-08-01T10:49:44.334Z</v>
+        <v>2026-08-08T07:13:24.089Z</v>
       </c>
       <c r="F392" t="str">
         <v>Success</v>
@@ -8253,7 +8253,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E393" t="str">
-        <v>2026-08-01T10:49:44.348Z</v>
+        <v>2026-08-08T07:13:24.104Z</v>
       </c>
       <c r="F393" t="str">
         <v>Success</v>
@@ -8270,10 +8270,10 @@
         <v>PASS</v>
       </c>
       <c r="D394" t="str">
-        <v>0.01 sec</v>
+        <v>0.02 sec</v>
       </c>
       <c r="E394" t="str">
-        <v>2026-08-01T10:49:44.363Z</v>
+        <v>2026-08-08T07:13:24.120Z</v>
       </c>
       <c r="F394" t="str">
         <v>Success</v>
@@ -8293,7 +8293,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E395" t="str">
-        <v>2026-08-01T10:49:44.378Z</v>
+        <v>2026-08-08T07:13:24.135Z</v>
       </c>
       <c r="F395" t="str">
         <v>Success</v>
@@ -8313,7 +8313,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E396" t="str">
-        <v>2026-08-01T10:49:44.394Z</v>
+        <v>2026-08-08T07:13:24.151Z</v>
       </c>
       <c r="F396" t="str">
         <v>Success</v>
@@ -8333,7 +8333,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E397" t="str">
-        <v>2026-08-01T10:49:44.409Z</v>
+        <v>2026-08-08T07:13:24.166Z</v>
       </c>
       <c r="F397" t="str">
         <v>Success</v>
@@ -8353,7 +8353,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E398" t="str">
-        <v>2026-08-01T10:49:44.425Z</v>
+        <v>2026-08-08T07:13:24.182Z</v>
       </c>
       <c r="F398" t="str">
         <v>Success</v>
@@ -8373,7 +8373,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E399" t="str">
-        <v>2026-08-01T10:49:44.440Z</v>
+        <v>2026-08-08T07:13:24.197Z</v>
       </c>
       <c r="F399" t="str">
         <v>Success</v>
@@ -8393,7 +8393,7 @@
         <v>0.02 sec</v>
       </c>
       <c r="E400" t="str">
-        <v>2026-08-01T10:49:44.456Z</v>
+        <v>2026-08-08T07:13:24.214Z</v>
       </c>
       <c r="F400" t="str">
         <v>Success</v>
@@ -8413,7 +8413,7 @@
         <v>0.01 sec</v>
       </c>
       <c r="E401" t="str">
-        <v>2026-08-01T10:49:44.471Z</v>
+        <v>2026-08-08T07:13:24.229Z</v>
       </c>
       <c r="F401" t="str">
         <v>Success</v>

</xml_diff>